<commit_message>
Remove unused legacy card group cleanup
</commit_message>
<xml_diff>
--- a/docs/testing/jira-miro-full-test-plan.xlsx
+++ b/docs/testing/jira-miro-full-test-plan.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testoversikt" sheetId="1" r:id="R96d3f70a26bb4861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testliste" sheetId="2" r:id="R3c9346e8514944de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dekning" sheetId="3" r:id="R3a130c53548a4ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testoversikt" sheetId="1" r:id="R0f7bc65093a946c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testliste" sheetId="2" r:id="Ra1e8adb59e2f4e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dekning" sheetId="3" r:id="R73e06116150a4f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funksjonsdekning" sheetId="4" r:id="R512d806e5df54e0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -211,7 +212,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="6">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -245,12 +246,45 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF216E39"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FullTestTable" displayName="FullTestTable" ref="A4:J68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FullTestTable" displayName="FullTestTable" ref="A4:J76" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Område"/>
@@ -529,16 +563,16 @@
         <x:v>Totalt antall tester</x:v>
       </x:c>
       <x:c r="B5" s="21" t="n">
-        <x:f>COUNTA(Testliste!$A$5:$A$68)</x:f>
-        <x:v>64</x:v>
+        <x:f>COUNTA(Testliste!$A$5:$A$76)</x:f>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="20" t="str">
         <x:v>Drift og sikkerhet</x:v>
       </x:c>
       <x:c r="E5" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$B$5:$B$68,"Drift og sikkerhet")</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTIF(Testliste!$B$5:$B$76,"Drift og sikkerhet")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F5" s="2"/>
       <x:c r="G5" s="2"/>
@@ -549,16 +583,16 @@
         <x:v>Bestått</x:v>
       </x:c>
       <x:c r="B6" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$G$5:$G$68,"Bestått")</x:f>
-        <x:v>56</x:v>
+        <x:f>COUNTIF(Testliste!$G$5:$G$76,"Bestått")</x:f>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="20" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="E6" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$B$5:$B$68,"Jira → Miro")</x:f>
-        <x:v>17</x:v>
+        <x:f>COUNTIF(Testliste!$B$5:$B$76,"Jira → Miro")</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F6" s="2"/>
       <x:c r="G6" s="2"/>
@@ -569,7 +603,7 @@
         <x:v>Feilet</x:v>
       </x:c>
       <x:c r="B7" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$G$5:$G$68,"Feilet")</x:f>
+        <x:f>COUNTIF(Testliste!$G$5:$G$76,"Feilet")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="2"/>
@@ -577,7 +611,7 @@
         <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="E7" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$B$5:$B$68,"Miro → Jira")</x:f>
+        <x:f>COUNTIF(Testliste!$B$5:$B$76,"Miro → Jira")</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="F7" s="2"/>
@@ -589,7 +623,7 @@
         <x:v>Blokkert</x:v>
       </x:c>
       <x:c r="B8" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$G$5:$G$68,"Blokkert")</x:f>
+        <x:f>COUNTIF(Testliste!$G$5:$G$76,"Blokkert")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
@@ -597,7 +631,7 @@
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="E8" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$B$5:$B$68,"Sticky → Jira")</x:f>
+        <x:f>COUNTIF(Testliste!$B$5:$B$76,"Sticky → Jira")</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="F8" s="2"/>
@@ -609,15 +643,15 @@
         <x:v>Ikke testet</x:v>
       </x:c>
       <x:c r="B9" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$G$5:$G$68,"Ikke testet")</x:f>
-        <x:v>4</x:v>
+        <x:f>COUNTIF(Testliste!$G$5:$G$76,"Ikke testet")</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="20" t="str">
         <x:v>Miro-app og UI</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
-        <x:f>COUNTIF(Testliste!$B$5:$B$68,"Miro-app og UI")</x:f>
+        <x:f>COUNTIF(Testliste!$B$5:$B$76,"Miro-app og UI")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F9" s="2"/>
@@ -629,7 +663,7 @@
         <x:v>Ikke relevant</x:v>
       </x:c>
       <x:c r="B10" s="23" t="n">
-        <x:f>COUNTIF(Testliste!$G$5:$G$68,"Ikke relevant")</x:f>
+        <x:f>COUNTIF(Testliste!$G$5:$G$76,"Ikke relevant")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
@@ -637,7 +671,7 @@
         <x:v>Reliabilitet</x:v>
       </x:c>
       <x:c r="E10" s="23" t="n">
-        <x:f>COUNTIF(Testliste!$B$5:$B$68,"Reliabilitet")</x:f>
+        <x:f>COUNTIF(Testliste!$B$5:$B$76,"Reliabilitet")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F10" s="2"/>
@@ -1082,22 +1116,22 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="14" t="str">
-        <x:v>B-01</x:v>
+        <x:v>A-06</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>Jira → Miro</x:v>
+        <x:v>Drift og sikkerhet</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
-        <x:v>Ny Jira-sak</x:v>
+        <x:v>Input-validering</x:v>
       </x:c>
       <x:c r="D10" s="4" t="str">
-        <x:v>Opprett en sak i Jira-prosjekt SN uten eksisterende Miro-mapping.</x:v>
+        <x:v>Send ugyldig JSON og webhook uten issueKey.</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
-        <x:v>Én custom Incoming-card opprettes. Ingen duplikat opprettes ved gjentatt webhook.</x:v>
+        <x:v>Ugyldig JSON avvises med 400. Webhook uten godkjent issueKey ignoreres trygt uten sideeffekt.</x:v>
       </x:c>
       <x:c r="F10" s="4" t="str">
-        <x:v>Miro-board og CARD_MAP</x:v>
+        <x:v>Ugyldig JSON: HTTP 400 og Invalid JSON. Manglende issueKey: ok:true, ignored:true, reason: Only SN issues are approved.</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1106,126 +1140,114 @@
         <x:v>Terje</x:v>
       </x:c>
       <x:c r="I10" s="5" t="n">
-        <x:v>46274.5</x:v>
+        <x:v>46275.25555555556</x:v>
       </x:c>
       <x:c r="J10" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Ingen Jira- eller Miro-endring.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="14" t="str">
-        <x:v>B-02</x:v>
+        <x:v>A-07</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>Jira → Miro</x:v>
+        <x:v>Drift og sikkerhet</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
-        <x:v>Eksisterende mapping</x:v>
+        <x:v>Board- og mapping-sikkerhet</x:v>
       </x:c>
       <x:c r="D11" s="4" t="str">
-        <x:v>Endre status på en Jira-sak som allerede har custom-card.</x:v>
+        <x:v>Send Miro-kall med feil boardId eller itemId som ikke er mappet til saken.</x:v>
       </x:c>
       <x:c r="E11" s="4" t="str">
-        <x:v>Riktig Miro-card flyttes. Ingen ny card opprettes.</x:v>
+        <x:v>Kallet avvises med 403 og ingen Jira-endring skjer.</x:v>
       </x:c>
       <x:c r="F11" s="4" t="str">
-        <x:v>Miro-board</x:v>
+        <x:v>HTTP-respons og Jira-status</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H11" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I11" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str"/>
+      <x:c r="I11" s="5" t="str"/>
       <x:c r="J11" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Funnet ved funksjonsaudit. Krever egen negativ test.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="14" t="str">
-        <x:v>B-03</x:v>
+        <x:v>A-08</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>Jira → Miro</x:v>
+        <x:v>Drift og sikkerhet</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
-        <x:v>Status Todo</x:v>
+        <x:v>Ukjent route/metode</x:v>
       </x:c>
       <x:c r="D12" s="4" t="str">
-        <x:v>Sett Jira-status til Todo.</x:v>
+        <x:v>Kall en ukjent route eller en route med feil HTTP-metode.</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
-        <x:v>Kortet ligger i Todo-kolonnen og Y-posisjon beholdes.</x:v>
+        <x:v>Worker svarer 404 uten sideeffekter.</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>Før/etter-posisjon</x:v>
+        <x:v>HTTP-respons</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H12" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I12" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="str"/>
+      <x:c r="I12" s="5" t="str"/>
       <x:c r="J12" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Funnet ved funksjonsaudit. Krever egen negativ test.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="14" t="str">
-        <x:v>B-04</x:v>
+        <x:v>A-09</x:v>
       </x:c>
       <x:c r="B13" s="3" t="str">
-        <x:v>Jira → Miro</x:v>
+        <x:v>Drift og sikkerhet</x:v>
       </x:c>
       <x:c r="C13" s="3" t="str">
-        <x:v>Status In Progress</x:v>
+        <x:v>Ugyldig status eller posisjon</x:v>
       </x:c>
       <x:c r="D13" s="4" t="str">
-        <x:v>Sett Jira-status til In Progress.</x:v>
+        <x:v>Send ugyldig issueKey, status eller kortposisjon til conversion-routes.</x:v>
       </x:c>
       <x:c r="E13" s="4" t="str">
-        <x:v>Kortet ligger i In Progress-kolonnen og Y-posisjon beholdes.</x:v>
+        <x:v>Kallet avvises kontrollert eller ignoreres uten duplikat eller sideeffekt.</x:v>
       </x:c>
       <x:c r="F13" s="4" t="str">
-        <x:v>Før/etter-posisjon</x:v>
+        <x:v>HTTP-respons og Miro-board</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H13" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I13" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="str"/>
+      <x:c r="I13" s="5" t="str"/>
       <x:c r="J13" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Funnet ved funksjonsaudit. Krever egen negativ test.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14" t="str">
-        <x:v>B-05</x:v>
+        <x:v>B-01</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
-        <x:v>Status Code Review</x:v>
+        <x:v>Ny Jira-sak</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:v>Sett Jira-status til Code Review.</x:v>
+        <x:v>Opprett en sak i Jira-prosjekt SN uten eksisterende Miro-mapping.</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
-        <x:v>Kortet ligger i Code Review-kolonnen og Y-posisjon beholdes.</x:v>
+        <x:v>Én custom Incoming-card opprettes. Ingen duplikat opprettes ved gjentatt webhook.</x:v>
       </x:c>
       <x:c r="F14" s="4" t="str">
-        <x:v>Før/etter-posisjon</x:v>
+        <x:v>Miro-board og CARD_MAP</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1242,22 +1264,22 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="14" t="str">
-        <x:v>B-06</x:v>
+        <x:v>B-02</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
-        <x:v>Status Functional Review</x:v>
+        <x:v>Eksisterende mapping</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>Sett Jira-status til Functional Review.</x:v>
+        <x:v>Endre status på en Jira-sak som allerede har custom-card.</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
-        <x:v>Kortet ligger i Functional Review-kolonnen og Y-posisjon beholdes.</x:v>
+        <x:v>Riktig Miro-card flyttes. Ingen ny card opprettes.</x:v>
       </x:c>
       <x:c r="F15" s="4" t="str">
-        <x:v>Før/etter-posisjon</x:v>
+        <x:v>Miro-board</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1274,19 +1296,19 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="14" t="str">
-        <x:v>B-07</x:v>
+        <x:v>B-03</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
-        <x:v>Status Done</x:v>
+        <x:v>Status Todo</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:v>Sett Jira-status til Done.</x:v>
+        <x:v>Sett Jira-status til Todo.</x:v>
       </x:c>
       <x:c r="E16" s="4" t="str">
-        <x:v>Kortet ligger i Done-kolonnen og Y-posisjon beholdes.</x:v>
+        <x:v>Kortet ligger i Todo-kolonnen og Y-posisjon beholdes.</x:v>
       </x:c>
       <x:c r="F16" s="4" t="str">
         <x:v>Før/etter-posisjon</x:v>
@@ -1306,22 +1328,22 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="14" t="str">
-        <x:v>B-08</x:v>
+        <x:v>B-04</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
-        <x:v>Status-only webhook</x:v>
+        <x:v>Status In Progress</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:v>Endre kun status i Jira.</x:v>
+        <x:v>Sett Jira-status til In Progress.</x:v>
       </x:c>
       <x:c r="E17" s="4" t="str">
-        <x:v>Kortet flyttes uten unødvendig SVG-refresh.</x:v>
+        <x:v>Kortet ligger i In Progress-kolonnen og Y-posisjon beholdes.</x:v>
       </x:c>
       <x:c r="F17" s="4" t="str">
-        <x:v>Cloudflare: webhook godkjent med 202, queue-behandling avsluttet uten feil. Detaljert refreshSkipped-logg er fjernet, så dette bekreftes også mot kortets innhold/utseende.</x:v>
+        <x:v>Før/etter-posisjon</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1332,26 +1354,28 @@
       <x:c r="I17" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J17" s="4" t="str"/>
+      <x:c r="J17" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="14" t="str">
-        <x:v>B-09</x:v>
+        <x:v>B-05</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
-        <x:v>Summary-refresh</x:v>
+        <x:v>Status Code Review</x:v>
       </x:c>
       <x:c r="D18" s="4" t="str">
-        <x:v>Endre Summary i Jira.</x:v>
+        <x:v>Sett Jira-status til Code Review.</x:v>
       </x:c>
       <x:c r="E18" s="4" t="str">
-        <x:v>Eksisterende custom-card oppdateres med ny tekst uten ny card.</x:v>
+        <x:v>Kortet ligger i Code Review-kolonnen og Y-posisjon beholdes.</x:v>
       </x:c>
       <x:c r="F18" s="4" t="str">
-        <x:v>Miro-card</x:v>
+        <x:v>Før/etter-posisjon</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1368,22 +1392,22 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="14" t="str">
-        <x:v>B-10</x:v>
+        <x:v>B-06</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
-        <x:v>Priority-refresh</x:v>
+        <x:v>Status Functional Review</x:v>
       </x:c>
       <x:c r="D19" s="4" t="str">
-        <x:v>Endre Priority i Jira.</x:v>
+        <x:v>Sett Jira-status til Functional Review.</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
-        <x:v>Eksisterende card oppdateres med riktig prioritetsvisning.</x:v>
+        <x:v>Kortet ligger i Functional Review-kolonnen og Y-posisjon beholdes.</x:v>
       </x:c>
       <x:c r="F19" s="4" t="str">
-        <x:v>Miro-card</x:v>
+        <x:v>Før/etter-posisjon</x:v>
       </x:c>
       <x:c r="G19" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1400,22 +1424,22 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="14" t="str">
-        <x:v>B-11</x:v>
+        <x:v>B-07</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C20" s="3" t="str">
-        <x:v>Assignee-refresh</x:v>
+        <x:v>Status Done</x:v>
       </x:c>
       <x:c r="D20" s="4" t="str">
-        <x:v>Endre Assignee i Jira.</x:v>
+        <x:v>Sett Jira-status til Done.</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
-        <x:v>Eksisterende card viser riktig assignee eller fallback.</x:v>
+        <x:v>Kortet ligger i Done-kolonnen og Y-posisjon beholdes.</x:v>
       </x:c>
       <x:c r="F20" s="4" t="str">
-        <x:v>Miro-card</x:v>
+        <x:v>Før/etter-posisjon</x:v>
       </x:c>
       <x:c r="G20" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1432,22 +1456,22 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14" t="str">
-        <x:v>B-12</x:v>
+        <x:v>B-08</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C21" s="3" t="str">
-        <x:v>Kommentarindikator</x:v>
+        <x:v>Status-only webhook</x:v>
       </x:c>
       <x:c r="D21" s="4" t="str">
-        <x:v>Legg til Jira-kommentar på en synket sak.</x:v>
+        <x:v>Endre kun status i Jira.</x:v>
       </x:c>
       <x:c r="E21" s="4" t="str">
-        <x:v>Kommentarindikator opprettes eller oppdateres med riktig antall.</x:v>
+        <x:v>Kortet flyttes uten unødvendig SVG-refresh.</x:v>
       </x:c>
       <x:c r="F21" s="4" t="str">
-        <x:v>Miro-board</x:v>
+        <x:v>Cloudflare: webhook godkjent med 202, queue-behandling avsluttet uten feil. Detaljert refreshSkipped-logg er fjernet, så dette bekreftes også mot kortets innhold/utseende.</x:v>
       </x:c>
       <x:c r="G21" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1458,28 +1482,26 @@
       <x:c r="I21" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J21" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
-      </x:c>
+      <x:c r="J21" s="4" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="14" t="str">
-        <x:v>B-13</x:v>
+        <x:v>B-09</x:v>
       </x:c>
       <x:c r="B22" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
-        <x:v>Kommentar slettes</x:v>
+        <x:v>Summary-refresh</x:v>
       </x:c>
       <x:c r="D22" s="4" t="str">
-        <x:v>Slett én av flere kommentarer og slett deretter alle kommentarer.</x:v>
+        <x:v>Endre Summary i Jira.</x:v>
       </x:c>
       <x:c r="E22" s="4" t="str">
-        <x:v>Indikatoren skal oppdateres til riktig antall og forsvinne når ingen kommentarer gjenstår.</x:v>
+        <x:v>Eksisterende custom-card oppdateres med ny tekst uten ny card.</x:v>
       </x:c>
       <x:c r="F22" s="4" t="str">
-        <x:v>Brev-ikonet oppdaterte antallet etter sletting og forsvant da siste kommentar ble slettet.</x:v>
+        <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G22" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1491,27 +1513,27 @@
         <x:v>46274.5</x:v>
       </x:c>
       <x:c r="J22" s="4" t="str">
-        <x:v>Jira comment_deleted-webhook lagt til og verifisert.</x:v>
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="14" t="str">
-        <x:v>B-14</x:v>
+        <x:v>B-10</x:v>
       </x:c>
       <x:c r="B23" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C23" s="3" t="str">
-        <x:v>Ukjent webhook-format</x:v>
+        <x:v>Priority-refresh</x:v>
       </x:c>
       <x:c r="D23" s="4" t="str">
-        <x:v>Send payload uten tydelig changedFields/changelog.</x:v>
+        <x:v>Endre Priority i Jira.</x:v>
       </x:c>
       <x:c r="E23" s="4" t="str">
-        <x:v>Full refresh brukes som fallback, og card blir korrekt oppdatert.</x:v>
+        <x:v>Eksisterende card oppdateres med riktig prioritetsvisning.</x:v>
       </x:c>
       <x:c r="F23" s="4" t="str">
-        <x:v>Webhook ble godtatt, full refresh gjennomført uten feil, og ingen duplikat-card oppstod.</x:v>
+        <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1522,26 +1544,28 @@
       <x:c r="I23" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J23" s="4" t="str"/>
+      <x:c r="J23" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="14" t="str">
-        <x:v>B-15</x:v>
+        <x:v>B-11</x:v>
       </x:c>
       <x:c r="B24" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C24" s="3" t="str">
-        <x:v>Mangler Miro-card</x:v>
+        <x:v>Assignee-refresh</x:v>
       </x:c>
       <x:c r="D24" s="4" t="str">
-        <x:v>Fjern eller ugyldiggjør en mapping og send statusendring.</x:v>
+        <x:v>Endre Assignee i Jira.</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
-        <x:v>Stale mapping håndteres, og én ny Incoming-card opprettes.</x:v>
+        <x:v>Eksisterende card viser riktig assignee eller fallback.</x:v>
       </x:c>
       <x:c r="F24" s="4" t="str">
-        <x:v>Stale mapping ble fjernet, ett nytt custom-kort ble opprettet i Incoming, og ingen duplikat oppstod.</x:v>
+        <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1552,26 +1576,28 @@
       <x:c r="I24" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J24" s="4" t="str"/>
+      <x:c r="J24" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="14" t="str">
-        <x:v>B-16</x:v>
+        <x:v>B-12</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C25" s="3" t="str">
-        <x:v>Retry etter feil</x:v>
+        <x:v>Kommentarindikator</x:v>
       </x:c>
       <x:c r="D25" s="4" t="str">
-        <x:v>Simuler eller fremprovoser midlertidig ekstern 5xx og la webhook retry.</x:v>
+        <x:v>Legg til Jira-kommentar på en synket sak.</x:v>
       </x:c>
       <x:c r="E25" s="4" t="str">
-        <x:v>Sync fullføres uten duplikat eller feil status.</x:v>
+        <x:v>Kommentarindikator opprettes eller oppdateres med riktig antall.</x:v>
       </x:c>
       <x:c r="F25" s="4" t="str">
-        <x:v>Cloudflare queue</x:v>
+        <x:v>Miro-board</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1588,22 +1614,22 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="14" t="str">
-        <x:v>B-17</x:v>
+        <x:v>B-13</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
         <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
-        <x:v>Rask gjentatt status</x:v>
+        <x:v>Kommentar slettes</x:v>
       </x:c>
       <x:c r="D26" s="4" t="str">
-        <x:v>Endre status to ganger innen 60 sekunder.</x:v>
+        <x:v>Slett én av flere kommentarer og slett deretter alle kommentarer.</x:v>
       </x:c>
       <x:c r="E26" s="4" t="str">
-        <x:v>Andre kall bruker validert parent-cache når samme Worker-instans brukes. Sync-resultatet er fortsatt korrekt.</x:v>
+        <x:v>Indikatoren skal oppdateres til riktig antall og forsvinne når ingen kommentarer gjenstår.</x:v>
       </x:c>
       <x:c r="F26" s="4" t="str">
-        <x:v>Cloudflare logs og Miro-board</x:v>
+        <x:v>Brev-ikonet oppdaterte antallet etter sletting og forsvant da siste kommentar ble slettet.</x:v>
       </x:c>
       <x:c r="G26" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1615,30 +1641,30 @@
         <x:v>46274.5</x:v>
       </x:c>
       <x:c r="J26" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Jira comment_deleted-webhook lagt til og verifisert.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="14" t="str">
-        <x:v>C-01</x:v>
+        <x:v>B-14</x:v>
       </x:c>
       <x:c r="B27" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C27" s="3" t="str">
-        <x:v>Native Jira-card drag</x:v>
+        <x:v>Ukjent webhook-format</x:v>
       </x:c>
       <x:c r="D27" s="4" t="str">
-        <x:v>Dra en native Jira-card til hver godkjente kolonne.</x:v>
+        <x:v>Send payload uten tydelig changedFields/changelog.</x:v>
       </x:c>
       <x:c r="E27" s="4" t="str">
-        <x:v>Jira-status følger kortets kolonne.</x:v>
+        <x:v>Full refresh brukes som fallback, og card blir korrekt oppdatert.</x:v>
       </x:c>
       <x:c r="F27" s="4" t="str">
-        <x:v>Ikke relevant: løsningen bruker kun custom cards.</x:v>
+        <x:v>Webhook ble godtatt, full refresh gjennomført uten feil, og ingen duplikat-card oppstod.</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
-        <x:v>Ikke relevant</x:v>
+        <x:v>Bestått</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
         <x:v>Terje</x:v>
@@ -1650,22 +1676,22 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="14" t="str">
-        <x:v>C-02</x:v>
+        <x:v>B-15</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C28" s="3" t="str">
-        <x:v>Custom-card drag</x:v>
+        <x:v>Mangler Miro-card</x:v>
       </x:c>
       <x:c r="D28" s="4" t="str">
-        <x:v>Dra en custom-card til hver godkjente kolonne.</x:v>
+        <x:v>Fjern eller ugyldiggjør en mapping og send statusendring.</x:v>
       </x:c>
       <x:c r="E28" s="4" t="str">
-        <x:v>Jira-status følger kortets kolonne.</x:v>
+        <x:v>Stale mapping håndteres, og én ny Incoming-card opprettes.</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
-        <x:v>Jira-status</x:v>
+        <x:v>Stale mapping ble fjernet, ett nytt custom-kort ble opprettet i Incoming, og ingen duplikat oppstod.</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1676,28 +1702,26 @@
       <x:c r="I28" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J28" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
-      </x:c>
+      <x:c r="J28" s="4" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="14" t="str">
-        <x:v>C-03</x:v>
+        <x:v>B-16</x:v>
       </x:c>
       <x:c r="B29" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C29" s="3" t="str">
-        <x:v>Under 60 prosent</x:v>
+        <x:v>Retry etter feil</x:v>
       </x:c>
       <x:c r="D29" s="4" t="str">
-        <x:v>Plasser kortet slik at ingen kolonne har minst 60 % overlap.</x:v>
+        <x:v>Simuler eller fremprovoser midlertidig ekstern 5xx og la webhook retry.</x:v>
       </x:c>
       <x:c r="E29" s="4" t="str">
-        <x:v>Ingen Jira-status endres.</x:v>
+        <x:v>Sync fullføres uten duplikat eller feil status.</x:v>
       </x:c>
       <x:c r="F29" s="4" t="str">
-        <x:v>Jira-status og Miro-posisjon</x:v>
+        <x:v>Cloudflare queue</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1714,22 +1738,22 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="14" t="str">
-        <x:v>C-04</x:v>
+        <x:v>B-17</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C30" s="3" t="str">
-        <x:v>På 60 prosent</x:v>
+        <x:v>Rask gjentatt status</x:v>
       </x:c>
       <x:c r="D30" s="4" t="str">
-        <x:v>Plasser kortet på grensen for 60 % overlap.</x:v>
+        <x:v>Endre status to ganger innen 60 sekunder.</x:v>
       </x:c>
       <x:c r="E30" s="4" t="str">
-        <x:v>Riktig kolonne velges og Jira-status oppdateres.</x:v>
+        <x:v>Andre kall bruker validert parent-cache når samme Worker-instans brukes. Sync-resultatet er fortsatt korrekt.</x:v>
       </x:c>
       <x:c r="F30" s="4" t="str">
-        <x:v>Jira-status</x:v>
+        <x:v>Cloudflare logs og Miro-board</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1746,153 +1770,137 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="14" t="str">
-        <x:v>C-05</x:v>
+        <x:v>B-18</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
-        <x:v>Y-posisjon ved Jira-sync</x:v>
+        <x:v>Blocker-prioritet</x:v>
       </x:c>
       <x:c r="D31" s="4" t="str">
-        <x:v>Dra kortet horisontalt mellom kolonner.</x:v>
+        <x:v>Sett Jira-prioritet til Blocker og la custom-card refreshe.</x:v>
       </x:c>
       <x:c r="E31" s="4" t="str">
-        <x:v>Jira-endringen flytter kortet tilbake til riktig kolonne uten uventet Y-endring.</x:v>
+        <x:v>Custom-card blir svart med hvit tekst, og Jira-lenken er fortsatt lesbar.</x:v>
       </x:c>
       <x:c r="F31" s="4" t="str">
-        <x:v>Før/etter-posisjon</x:v>
+        <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H31" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I31" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H31" s="3" t="str"/>
+      <x:c r="I31" s="5" t="str"/>
       <x:c r="J31" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Funnet ved funksjonsaudit. Krever egen visuell test.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="14" t="str">
-        <x:v>C-06</x:v>
+        <x:v>B-19</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C32" s="3" t="str">
-        <x:v>Utenfor workflow</x:v>
+        <x:v>Hotfix-felt</x:v>
       </x:c>
       <x:c r="D32" s="4" t="str">
-        <x:v>Dra kortet utenfor workflow-området.</x:v>
+        <x:v>Aktiver hotfix-feltet på en Jira-sak og la custom-card refreshe.</x:v>
       </x:c>
       <x:c r="E32" s="4" t="str">
-        <x:v>Ingen ugyldig status sendes til Jira.</x:v>
+        <x:v>Custom-card blir oransje og beholder riktig innhold, lenke og mapping.</x:v>
       </x:c>
       <x:c r="F32" s="4" t="str">
-        <x:v>Jira-status</x:v>
+        <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G32" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H32" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I32" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H32" s="3" t="str"/>
+      <x:c r="I32" s="5" t="str"/>
       <x:c r="J32" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Funnet ved funksjonsaudit. Krever egen visuell test.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="14" t="str">
-        <x:v>C-07</x:v>
+        <x:v>B-20</x:v>
       </x:c>
       <x:c r="B33" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C33" s="3" t="str">
-        <x:v>Jira-avvisning og rollback</x:v>
+        <x:v>Work type-farger</x:v>
       </x:c>
       <x:c r="D33" s="4" t="str">
-        <x:v>Utfør en overgang Jira skal avvise.</x:v>
+        <x:v>Kontroller custom-card for Bug, Improvement, Spike, New Feature og Task/config/doc/test.</x:v>
       </x:c>
       <x:c r="E33" s="4" t="str">
-        <x:v>Kortet rulles tilbake til forrige posisjon og bruker får feilmelding.</x:v>
+        <x:v>Kortet bruker riktig farge for hver work type.</x:v>
       </x:c>
       <x:c r="F33" s="4" t="str">
-        <x:v>Miro-board og UI</x:v>
+        <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G33" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H33" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I33" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H33" s="3" t="str"/>
+      <x:c r="I33" s="5" t="str"/>
       <x:c r="J33" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Funnet ved funksjonsaudit. Krever egen visuell test.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="14" t="str">
-        <x:v>C-08</x:v>
+        <x:v>B-21</x:v>
       </x:c>
       <x:c r="B34" s="3" t="str">
-        <x:v>Miro → Jira</x:v>
+        <x:v>Jira → Miro</x:v>
       </x:c>
       <x:c r="C34" s="3" t="str">
-        <x:v>Functional Review uten Test area</x:v>
+        <x:v>Prioritetsikoner</x:v>
       </x:c>
       <x:c r="D34" s="4" t="str">
-        <x:v>Forsøk å flytte til Functional Review med tomt Test area-felt.</x:v>
+        <x:v>Kontroller custom-card med Blocker, Highest, High, Medium, Low, Lowest og uten prioritet.</x:v>
       </x:c>
       <x:c r="E34" s="4" t="str">
-        <x:v>Jira avviser overgangen, Miro rulles tilbake, og tydelig melding vises.</x:v>
+        <x:v>Riktig prioritetsikon og prioritetstekst vises for hver verdi.</x:v>
       </x:c>
       <x:c r="F34" s="4" t="str">
-        <x:v>Jira og Miro UI</x:v>
+        <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H34" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I34" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H34" s="3" t="str"/>
+      <x:c r="I34" s="5" t="str"/>
       <x:c r="J34" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Funnet ved funksjonsaudit. Krever egen visuell test.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="14" t="str">
-        <x:v>C-09</x:v>
+        <x:v>C-01</x:v>
       </x:c>
       <x:c r="B35" s="3" t="str">
         <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C35" s="3" t="str">
-        <x:v>Functional Review med Test area</x:v>
+        <x:v>Native Jira-card drag</x:v>
       </x:c>
       <x:c r="D35" s="4" t="str">
-        <x:v>Fyll Test area og flytt til Functional Review.</x:v>
+        <x:v>Dra en native Jira-card til hver godkjente kolonne.</x:v>
       </x:c>
       <x:c r="E35" s="4" t="str">
-        <x:v>Overgangen godtas og kortet blir stående i riktig kolonne.</x:v>
+        <x:v>Jira-status følger kortets kolonne.</x:v>
       </x:c>
       <x:c r="F35" s="4" t="str">
-        <x:v>Jira og Miro UI</x:v>
+        <x:v>Ikke relevant: løsningen bruker kun custom cards.</x:v>
       </x:c>
       <x:c r="G35" s="3" t="str">
-        <x:v>Bestått</x:v>
+        <x:v>Ikke relevant</x:v>
       </x:c>
       <x:c r="H35" s="3" t="str">
         <x:v>Terje</x:v>
@@ -1900,28 +1908,26 @@
       <x:c r="I35" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J35" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
-      </x:c>
+      <x:c r="J35" s="4" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="14" t="str">
-        <x:v>C-10</x:v>
+        <x:v>C-02</x:v>
       </x:c>
       <x:c r="B36" s="3" t="str">
         <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C36" s="3" t="str">
-        <x:v>Kollisjon mellom kort</x:v>
+        <x:v>Custom-card drag</x:v>
       </x:c>
       <x:c r="D36" s="4" t="str">
-        <x:v>Flytt et kort til en kolonne der målposisjonen er opptatt.</x:v>
+        <x:v>Dra en custom-card til hver godkjente kolonne.</x:v>
       </x:c>
       <x:c r="E36" s="4" t="str">
-        <x:v>Kortet plasseres innenfor kolonnen uten å dekke et annet Jira-kort.</x:v>
+        <x:v>Jira-status følger kortets kolonne.</x:v>
       </x:c>
       <x:c r="F36" s="4" t="str">
-        <x:v>Miro-board</x:v>
+        <x:v>Jira-status</x:v>
       </x:c>
       <x:c r="G36" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1938,22 +1944,22 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="14" t="str">
-        <x:v>C-11</x:v>
+        <x:v>C-03</x:v>
       </x:c>
       <x:c r="B37" s="3" t="str">
         <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C37" s="3" t="str">
-        <x:v>Debounce</x:v>
+        <x:v>Under 60 prosent</x:v>
       </x:c>
       <x:c r="D37" s="4" t="str">
-        <x:v>Dra samme kort flere ganger raskt.</x:v>
+        <x:v>Plasser kortet slik at ingen kolonne har minst 60 % overlap.</x:v>
       </x:c>
       <x:c r="E37" s="4" t="str">
-        <x:v>Kun siste stabile posisjon behandles, og ingen ekstra feilstatus sendes.</x:v>
+        <x:v>Ingen Jira-status endres.</x:v>
       </x:c>
       <x:c r="F37" s="4" t="str">
-        <x:v>Jira-status og nettverk</x:v>
+        <x:v>Jira-status og Miro-posisjon</x:v>
       </x:c>
       <x:c r="G37" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -1970,22 +1976,22 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="14" t="str">
-        <x:v>C-12</x:v>
+        <x:v>C-04</x:v>
       </x:c>
       <x:c r="B38" s="3" t="str">
         <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C38" s="3" t="str">
-        <x:v>Kommentarer åpnes</x:v>
+        <x:v>På 60 prosent</x:v>
       </x:c>
       <x:c r="D38" s="4" t="str">
-        <x:v>Klikk kommentarindikator eller kortmeny og åpne kommentarer.</x:v>
+        <x:v>Plasser kortet på grensen for 60 % overlap.</x:v>
       </x:c>
       <x:c r="E38" s="4" t="str">
-        <x:v>Modal åpnes og viser riktige Jira-kommentarer.</x:v>
+        <x:v>Riktig kolonne velges og Jira-status oppdateres.</x:v>
       </x:c>
       <x:c r="F38" s="4" t="str">
-        <x:v>Miro UI</x:v>
+        <x:v>Jira-status</x:v>
       </x:c>
       <x:c r="G38" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2002,22 +2008,22 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="14" t="str">
-        <x:v>C-13</x:v>
+        <x:v>C-05</x:v>
       </x:c>
       <x:c r="B39" s="3" t="str">
         <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C39" s="3" t="str">
-        <x:v>Ny Miro-kommentar</x:v>
+        <x:v>Y-posisjon ved Jira-sync</x:v>
       </x:c>
       <x:c r="D39" s="4" t="str">
-        <x:v>Skriv og send kommentar fra Miro.</x:v>
+        <x:v>Dra kortet horisontalt mellom kolonner.</x:v>
       </x:c>
       <x:c r="E39" s="4" t="str">
-        <x:v>Kommentaren opprettes i riktig Jira-sak.</x:v>
+        <x:v>Jira-endringen flytter kortet tilbake til riktig kolonne uten uventet Y-endring.</x:v>
       </x:c>
       <x:c r="F39" s="4" t="str">
-        <x:v>Jira-kommentar</x:v>
+        <x:v>Før/etter-posisjon</x:v>
       </x:c>
       <x:c r="G39" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2034,22 +2040,22 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="14" t="str">
-        <x:v>D-01</x:v>
+        <x:v>C-06</x:v>
       </x:c>
       <x:c r="B40" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C40" s="3" t="str">
-        <x:v>Én sticky utenfor workflow</x:v>
+        <x:v>Utenfor workflow</x:v>
       </x:c>
       <x:c r="D40" s="4" t="str">
-        <x:v>Velg én sticky utenfor workflow og konverter.</x:v>
+        <x:v>Dra kortet utenfor workflow-området.</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
-        <x:v>Én Jira-sak opprettes med default-status, custom-card opprettes på eksakt posisjon, sticky fjernes etter suksess.</x:v>
+        <x:v>Ingen ugyldig status sendes til Jira.</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
-        <x:v>Jira og Miro-board</x:v>
+        <x:v>Jira-status</x:v>
       </x:c>
       <x:c r="G40" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2066,22 +2072,22 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="14" t="str">
-        <x:v>D-02</x:v>
+        <x:v>C-07</x:v>
       </x:c>
       <x:c r="B41" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C41" s="3" t="str">
-        <x:v>Sticky i Todo</x:v>
+        <x:v>Jira-avvisning og rollback</x:v>
       </x:c>
       <x:c r="D41" s="4" t="str">
-        <x:v>Konverter sticky plassert i Todo-kolonnen.</x:v>
+        <x:v>Utfør en overgang Jira skal avvise.</x:v>
       </x:c>
       <x:c r="E41" s="4" t="str">
-        <x:v>Jira-sak får Todo-status og card beholder eksakt posisjon.</x:v>
+        <x:v>Kortet rulles tilbake til forrige posisjon og bruker får feilmelding.</x:v>
       </x:c>
       <x:c r="F41" s="4" t="str">
-        <x:v>Jira og Miro-board</x:v>
+        <x:v>Miro-board og UI</x:v>
       </x:c>
       <x:c r="G41" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2098,22 +2104,22 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="14" t="str">
-        <x:v>D-03</x:v>
+        <x:v>C-08</x:v>
       </x:c>
       <x:c r="B42" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C42" s="3" t="str">
-        <x:v>Sticky i In Progress</x:v>
+        <x:v>Functional Review uten Test area</x:v>
       </x:c>
       <x:c r="D42" s="4" t="str">
-        <x:v>Konverter sticky plassert i In Progress-kolonnen.</x:v>
+        <x:v>Forsøk å flytte til Functional Review med tomt Test area-felt.</x:v>
       </x:c>
       <x:c r="E42" s="4" t="str">
-        <x:v>Jira-sak får In Progress-status.</x:v>
+        <x:v>Jira avviser overgangen, Miro rulles tilbake, og tydelig melding vises.</x:v>
       </x:c>
       <x:c r="F42" s="4" t="str">
-        <x:v>Jira og Miro-board</x:v>
+        <x:v>Jira og Miro UI</x:v>
       </x:c>
       <x:c r="G42" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2130,22 +2136,22 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="14" t="str">
-        <x:v>D-04</x:v>
+        <x:v>C-09</x:v>
       </x:c>
       <x:c r="B43" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C43" s="3" t="str">
-        <x:v>Sticky i Code Review</x:v>
+        <x:v>Functional Review med Test area</x:v>
       </x:c>
       <x:c r="D43" s="4" t="str">
-        <x:v>Konverter sticky plassert i Code Review-kolonnen.</x:v>
+        <x:v>Fyll Test area og flytt til Functional Review.</x:v>
       </x:c>
       <x:c r="E43" s="4" t="str">
-        <x:v>Jira-sak får Code Review-status.</x:v>
+        <x:v>Overgangen godtas og kortet blir stående i riktig kolonne.</x:v>
       </x:c>
       <x:c r="F43" s="4" t="str">
-        <x:v>Jira og Miro-board</x:v>
+        <x:v>Jira og Miro UI</x:v>
       </x:c>
       <x:c r="G43" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2162,22 +2168,22 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="14" t="str">
-        <x:v>D-05</x:v>
+        <x:v>C-10</x:v>
       </x:c>
       <x:c r="B44" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C44" s="3" t="str">
-        <x:v>Sticky i Functional Review</x:v>
+        <x:v>Kollisjon mellom kort</x:v>
       </x:c>
       <x:c r="D44" s="4" t="str">
-        <x:v>Konverter sticky plassert i Functional Review med Test area tilgjengelig.</x:v>
+        <x:v>Flytt et kort til en kolonne der målposisjonen er opptatt.</x:v>
       </x:c>
       <x:c r="E44" s="4" t="str">
-        <x:v>Jira-sak får Functional Review-status.</x:v>
+        <x:v>Kortet plasseres innenfor kolonnen uten å dekke et annet Jira-kort.</x:v>
       </x:c>
       <x:c r="F44" s="4" t="str">
-        <x:v>Jira og Miro-board</x:v>
+        <x:v>Miro-board</x:v>
       </x:c>
       <x:c r="G44" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2194,22 +2200,22 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="14" t="str">
-        <x:v>D-06</x:v>
+        <x:v>C-11</x:v>
       </x:c>
       <x:c r="B45" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C45" s="3" t="str">
-        <x:v>Sticky i Done</x:v>
+        <x:v>Debounce</x:v>
       </x:c>
       <x:c r="D45" s="4" t="str">
-        <x:v>Konverter sticky plassert i Done-kolonnen.</x:v>
+        <x:v>Dra samme kort flere ganger raskt.</x:v>
       </x:c>
       <x:c r="E45" s="4" t="str">
-        <x:v>Jira-sak får Done-status.</x:v>
+        <x:v>Kun siste stabile posisjon behandles, og ingen ekstra feilstatus sendes.</x:v>
       </x:c>
       <x:c r="F45" s="4" t="str">
-        <x:v>Jira og Miro-board</x:v>
+        <x:v>Jira-status og nettverk</x:v>
       </x:c>
       <x:c r="G45" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2226,22 +2232,22 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="14" t="str">
-        <x:v>D-07</x:v>
+        <x:v>C-12</x:v>
       </x:c>
       <x:c r="B46" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C46" s="3" t="str">
-        <x:v>Work type Bug</x:v>
+        <x:v>Kommentarer åpnes</x:v>
       </x:c>
       <x:c r="D46" s="4" t="str">
-        <x:v>Konverter en sticky med Bug-farge.</x:v>
+        <x:v>Klikk kommentarindikator eller kortmeny og åpne kommentarer.</x:v>
       </x:c>
       <x:c r="E46" s="4" t="str">
-        <x:v>Jira-sak opprettes som Bug med riktige defaults.</x:v>
+        <x:v>Modal åpnes og viser riktige Jira-kommentarer.</x:v>
       </x:c>
       <x:c r="F46" s="4" t="str">
-        <x:v>Jira-sak</x:v>
+        <x:v>Miro UI</x:v>
       </x:c>
       <x:c r="G46" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2258,22 +2264,22 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="14" t="str">
-        <x:v>D-08</x:v>
+        <x:v>C-13</x:v>
       </x:c>
       <x:c r="B47" s="3" t="str">
-        <x:v>Sticky → Jira</x:v>
+        <x:v>Miro → Jira</x:v>
       </x:c>
       <x:c r="C47" s="3" t="str">
-        <x:v>Work type Improvement</x:v>
+        <x:v>Ny Miro-kommentar</x:v>
       </x:c>
       <x:c r="D47" s="4" t="str">
-        <x:v>Konverter en sticky med Improvement-farge.</x:v>
+        <x:v>Skriv og send kommentar fra Miro.</x:v>
       </x:c>
       <x:c r="E47" s="4" t="str">
-        <x:v>Jira-sak opprettes som Improvement med riktige defaults.</x:v>
+        <x:v>Kommentaren opprettes i riktig Jira-sak.</x:v>
       </x:c>
       <x:c r="F47" s="4" t="str">
-        <x:v>Jira-sak</x:v>
+        <x:v>Jira-kommentar</x:v>
       </x:c>
       <x:c r="G47" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2290,22 +2296,22 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="14" t="str">
-        <x:v>D-09</x:v>
+        <x:v>D-01</x:v>
       </x:c>
       <x:c r="B48" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C48" s="3" t="str">
-        <x:v>Work type New Feature</x:v>
+        <x:v>Én sticky utenfor workflow</x:v>
       </x:c>
       <x:c r="D48" s="4" t="str">
-        <x:v>Konverter en sticky med New Feature-farge.</x:v>
+        <x:v>Velg én sticky utenfor workflow og konverter.</x:v>
       </x:c>
       <x:c r="E48" s="4" t="str">
-        <x:v>Jira-sak opprettes som New Feature med riktige defaults.</x:v>
+        <x:v>Én Jira-sak opprettes med default-status, custom-card opprettes på eksakt posisjon, sticky fjernes etter suksess.</x:v>
       </x:c>
       <x:c r="F48" s="4" t="str">
-        <x:v>Jira-sak</x:v>
+        <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G48" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2322,22 +2328,22 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="14" t="str">
-        <x:v>D-10</x:v>
+        <x:v>D-02</x:v>
       </x:c>
       <x:c r="B49" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C49" s="3" t="str">
-        <x:v>Work type Task/config/doc/test</x:v>
+        <x:v>Sticky i Todo</x:v>
       </x:c>
       <x:c r="D49" s="4" t="str">
-        <x:v>Konverter sticky som skal bli Task/config/doc/test.</x:v>
+        <x:v>Konverter sticky plassert i Todo-kolonnen.</x:v>
       </x:c>
       <x:c r="E49" s="4" t="str">
-        <x:v>Riktig work type og obligatoriske felter brukes.</x:v>
+        <x:v>Jira-sak får Todo-status og card beholder eksakt posisjon.</x:v>
       </x:c>
       <x:c r="F49" s="4" t="str">
-        <x:v>Jira-sak</x:v>
+        <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G49" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2354,22 +2360,22 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="14" t="str">
-        <x:v>D-11</x:v>
+        <x:v>D-03</x:v>
       </x:c>
       <x:c r="B50" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C50" s="3" t="str">
-        <x:v>Reporter</x:v>
+        <x:v>Sticky i In Progress</x:v>
       </x:c>
       <x:c r="D50" s="4" t="str">
-        <x:v>Konverter sticky opprettet av kjent Miro-bruker.</x:v>
+        <x:v>Konverter sticky plassert i In Progress-kolonnen.</x:v>
       </x:c>
       <x:c r="E50" s="4" t="str">
-        <x:v>Riktig Jira Reporter settes, med cache ved senere konvertering.</x:v>
+        <x:v>Jira-sak får In Progress-status.</x:v>
       </x:c>
       <x:c r="F50" s="4" t="str">
-        <x:v>Jira-sak</x:v>
+        <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G50" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2386,22 +2392,22 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="14" t="str">
-        <x:v>D-12</x:v>
+        <x:v>D-04</x:v>
       </x:c>
       <x:c r="B51" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C51" s="3" t="str">
-        <x:v>Original Miro created</x:v>
+        <x:v>Sticky i Code Review</x:v>
       </x:c>
       <x:c r="D51" s="4" t="str">
-        <x:v>Konverter sticky og kontroller metadatafeltet.</x:v>
+        <x:v>Konverter sticky plassert i Code Review-kolonnen.</x:v>
       </x:c>
       <x:c r="E51" s="4" t="str">
-        <x:v>Original Miro-opprettelsestidspunkt lagres i Jira.</x:v>
+        <x:v>Jira-sak får Code Review-status.</x:v>
       </x:c>
       <x:c r="F51" s="4" t="str">
-        <x:v>Jira-sak</x:v>
+        <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G51" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2418,74 +2424,86 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="14" t="str">
-        <x:v>D-13</x:v>
+        <x:v>D-05</x:v>
       </x:c>
       <x:c r="B52" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C52" s="3" t="str">
-        <x:v>Idempotent retry</x:v>
+        <x:v>Sticky i Functional Review</x:v>
       </x:c>
       <x:c r="D52" s="4" t="str">
-        <x:v>Avbryt etter Jira-opprettelse og kjør samme konvertering på nytt.</x:v>
+        <x:v>Konverter sticky plassert i Functional Review med Test area tilgjengelig.</x:v>
       </x:c>
       <x:c r="E52" s="4" t="str">
-        <x:v>Samme Jira-sak gjenbrukes. Ingen duplikat opprettes.</x:v>
+        <x:v>Jira-sak får Functional Review-status.</x:v>
       </x:c>
       <x:c r="F52" s="4" t="str">
         <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G52" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H52" s="3" t="str"/>
-      <x:c r="I52" s="5" t="str"/>
-      <x:c r="J52" s="4" t="str"/>
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H52" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I52" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J52" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="14" t="str">
-        <x:v>D-14</x:v>
+        <x:v>D-06</x:v>
       </x:c>
       <x:c r="B53" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C53" s="3" t="str">
-        <x:v>Sticky fjernes først etter suksess</x:v>
+        <x:v>Sticky i Done</x:v>
       </x:c>
       <x:c r="D53" s="4" t="str">
-        <x:v>Simuler feil ved card-opprettelse eller Jira-overgang.</x:v>
+        <x:v>Konverter sticky plassert i Done-kolonnen.</x:v>
       </x:c>
       <x:c r="E53" s="4" t="str">
-        <x:v>Sticky beholdes, og brukeren får feilmelding.</x:v>
+        <x:v>Jira-sak får Done-status.</x:v>
       </x:c>
       <x:c r="F53" s="4" t="str">
-        <x:v>Miro-board og UI</x:v>
+        <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G53" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H53" s="3" t="str"/>
-      <x:c r="I53" s="5" t="str"/>
-      <x:c r="J53" s="4" t="str"/>
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H53" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I53" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J53" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="14" t="str">
-        <x:v>D-15</x:v>
+        <x:v>D-07</x:v>
       </x:c>
       <x:c r="B54" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C54" s="3" t="str">
-        <x:v>Multi-select</x:v>
+        <x:v>Work type Bug</x:v>
       </x:c>
       <x:c r="D54" s="4" t="str">
-        <x:v>Velg flere stickies der én har feil data.</x:v>
+        <x:v>Konverter en sticky med Bug-farge.</x:v>
       </x:c>
       <x:c r="E54" s="4" t="str">
-        <x:v>Gyldige stickies konverteres, og én feil stopper ikke resten.</x:v>
+        <x:v>Jira-sak opprettes som Bug med riktige defaults.</x:v>
       </x:c>
       <x:c r="F54" s="4" t="str">
-        <x:v>Jira og Miro-board</x:v>
+        <x:v>Jira-sak</x:v>
       </x:c>
       <x:c r="G54" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2502,22 +2520,22 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="14" t="str">
-        <x:v>D-16</x:v>
+        <x:v>D-08</x:v>
       </x:c>
       <x:c r="B55" s="3" t="str">
         <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C55" s="3" t="str">
-        <x:v>Direkte Jira-sak samtidig</x:v>
+        <x:v>Work type Improvement</x:v>
       </x:c>
       <x:c r="D55" s="4" t="str">
-        <x:v>Opprett Jira-sak direkte mens sticky-konvertering skjer.</x:v>
+        <x:v>Konverter en sticky med Improvement-farge.</x:v>
       </x:c>
       <x:c r="E55" s="4" t="str">
-        <x:v>Direkte Jira-sak går til Incoming; sticky-opprinnelig sak lager ikke ekstra Incoming-card.</x:v>
+        <x:v>Jira-sak opprettes som Improvement med riktige defaults.</x:v>
       </x:c>
       <x:c r="F55" s="4" t="str">
-        <x:v>Miro-board</x:v>
+        <x:v>Jira-sak</x:v>
       </x:c>
       <x:c r="G55" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2534,22 +2552,22 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="14" t="str">
-        <x:v>E-01</x:v>
+        <x:v>D-09</x:v>
       </x:c>
       <x:c r="B56" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C56" s="3" t="str">
-        <x:v>App åpnes</x:v>
+        <x:v>Work type New Feature</x:v>
       </x:c>
       <x:c r="D56" s="4" t="str">
-        <x:v>Åpne Miro-appen og klikk appikon/panel.</x:v>
+        <x:v>Konverter en sticky med New Feature-farge.</x:v>
       </x:c>
       <x:c r="E56" s="4" t="str">
-        <x:v>Panel åpnes, eksisterende kort oppdages, og /health er tilgjengelig.</x:v>
+        <x:v>Jira-sak opprettes som New Feature med riktige defaults.</x:v>
       </x:c>
       <x:c r="F56" s="4" t="str">
-        <x:v>Miro UI</x:v>
+        <x:v>Jira-sak</x:v>
       </x:c>
       <x:c r="G56" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2566,22 +2584,22 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="14" t="str">
-        <x:v>E-02</x:v>
+        <x:v>D-10</x:v>
       </x:c>
       <x:c r="B57" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C57" s="3" t="str">
-        <x:v>Custom-card registrering</x:v>
+        <x:v>Work type Task/config/doc/test</x:v>
       </x:c>
       <x:c r="D57" s="4" t="str">
-        <x:v>Åpne board med eksisterende custom cards.</x:v>
+        <x:v>Konverter sticky som skal bli Task/config/doc/test.</x:v>
       </x:c>
       <x:c r="E57" s="4" t="str">
-        <x:v>Custom-card Jira-lenker og mappings registreres uten duplikat.</x:v>
+        <x:v>Riktig work type og obligatoriske felter brukes.</x:v>
       </x:c>
       <x:c r="F57" s="4" t="str">
-        <x:v>Miro-board og CARD_MAP</x:v>
+        <x:v>Jira-sak</x:v>
       </x:c>
       <x:c r="G57" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2598,25 +2616,25 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="14" t="str">
-        <x:v>E-03</x:v>
+        <x:v>D-11</x:v>
       </x:c>
       <x:c r="B58" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C58" s="3" t="str">
-        <x:v>Jira-link på native-card</x:v>
+        <x:v>Reporter</x:v>
       </x:c>
       <x:c r="D58" s="4" t="str">
-        <x:v>Klikk Jira-lenken på et native Jira-kort.</x:v>
+        <x:v>Konverter sticky opprettet av kjent Miro-bruker.</x:v>
       </x:c>
       <x:c r="E58" s="4" t="str">
-        <x:v>Lenken åpner riktig Jira-sak i riktig site/prosjekt.</x:v>
+        <x:v>Riktig Jira Reporter settes, med cache ved senere konvertering.</x:v>
       </x:c>
       <x:c r="F58" s="4" t="str">
-        <x:v>Ikke relevant: løsningen bruker kun custom cards.</x:v>
+        <x:v>Jira-sak</x:v>
       </x:c>
       <x:c r="G58" s="3" t="str">
-        <x:v>Ikke relevant</x:v>
+        <x:v>Bestått</x:v>
       </x:c>
       <x:c r="H58" s="3" t="str">
         <x:v>Terje</x:v>
@@ -2624,26 +2642,28 @@
       <x:c r="I58" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J58" s="4" t="str"/>
+      <x:c r="J58" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="14" t="str">
-        <x:v>E-04</x:v>
+        <x:v>D-12</x:v>
       </x:c>
       <x:c r="B59" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C59" s="3" t="str">
-        <x:v>Jira-link på custom-card</x:v>
+        <x:v>Original Miro created</x:v>
       </x:c>
       <x:c r="D59" s="4" t="str">
-        <x:v>Klikk Jira-lenken på et custom-kort.</x:v>
+        <x:v>Konverter sticky og kontroller metadatafeltet.</x:v>
       </x:c>
       <x:c r="E59" s="4" t="str">
-        <x:v>Lenken åpner riktig Jira-sak i riktig site/prosjekt.</x:v>
+        <x:v>Original Miro-opprettelsestidspunkt lagres i Jira.</x:v>
       </x:c>
       <x:c r="F59" s="4" t="str">
-        <x:v>Nettleser og Jira-URL</x:v>
+        <x:v>Jira-sak</x:v>
       </x:c>
       <x:c r="G59" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2660,87 +2680,77 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="14" t="str">
-        <x:v>E-05</x:v>
+        <x:v>D-13</x:v>
       </x:c>
       <x:c r="B60" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C60" s="3" t="str">
-        <x:v>Jira-link etter refresh</x:v>
+        <x:v>Idempotent retry</x:v>
       </x:c>
       <x:c r="D60" s="4" t="str">
-        <x:v>Refresh Miro, åpne boardet på nytt og klikk lenken på et custom-kort.</x:v>
+        <x:v>Avbryt etter Jira-opprettelse og kjør samme konvertering på nytt.</x:v>
       </x:c>
       <x:c r="E60" s="4" t="str">
-        <x:v>Lenken er fortsatt til stede og peker til riktig Jira-sak.</x:v>
+        <x:v>Samme Jira-sak gjenbrukes. Ingen duplikat opprettes.</x:v>
       </x:c>
       <x:c r="F60" s="4" t="str">
-        <x:v>Miro-board og Jira-URL</x:v>
+        <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G60" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H60" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I60" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
-      <x:c r="J60" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H60" s="3" t="str"/>
+      <x:c r="I60" s="5" t="str"/>
+      <x:c r="J60" s="4" t="str"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="14" t="str">
-        <x:v>E-06</x:v>
+        <x:v>D-14</x:v>
       </x:c>
       <x:c r="B61" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C61" s="3" t="str">
-        <x:v>Legacy group-opprydding</x:v>
+        <x:v>Sticky fjernes først etter suksess</x:v>
       </x:c>
       <x:c r="D61" s="4" t="str">
-        <x:v>Test av gammel native-card/grupperingslogikk.</x:v>
+        <x:v>Simuler feil ved card-opprettelse eller Jira-overgang.</x:v>
       </x:c>
       <x:c r="E61" s="4" t="str">
-        <x:v>Ikke relevant: løsningen bruker kun custom cards.</x:v>
+        <x:v>Sticky beholdes, og brukeren får feilmelding.</x:v>
       </x:c>
       <x:c r="F61" s="4" t="str">
-        <x:v>Ikke relevant: native Jira cards brukes ikke.</x:v>
+        <x:v>Miro-board og UI</x:v>
       </x:c>
       <x:c r="G61" s="3" t="str">
-        <x:v>Ikke relevant</x:v>
-      </x:c>
-      <x:c r="H61" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I61" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H61" s="3" t="str"/>
+      <x:c r="I61" s="5" t="str"/>
       <x:c r="J61" s="4" t="str"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="14" t="str">
-        <x:v>E-07</x:v>
+        <x:v>D-15</x:v>
       </x:c>
       <x:c r="B62" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C62" s="3" t="str">
-        <x:v>Kommentarindikator følger kort</x:v>
+        <x:v>Multi-select</x:v>
       </x:c>
       <x:c r="D62" s="4" t="str">
-        <x:v>Test av gammel kort-/indikatorflyt.</x:v>
+        <x:v>Velg flere stickies der én har feil data.</x:v>
       </x:c>
       <x:c r="E62" s="4" t="str">
-        <x:v>Ikke relevant: denne flyten inngår ikke i ønsket custom-card-testomfang.</x:v>
+        <x:v>Gyldige stickies konverteres, og én feil stopper ikke resten.</x:v>
       </x:c>
       <x:c r="F62" s="4" t="str">
-        <x:v>Ikke relevant: utenfor avtalt testomfang.</x:v>
+        <x:v>Jira og Miro-board</x:v>
       </x:c>
       <x:c r="G62" s="3" t="str">
-        <x:v>Ikke relevant</x:v>
+        <x:v>Bestått</x:v>
       </x:c>
       <x:c r="H62" s="3" t="str">
         <x:v>Terje</x:v>
@@ -2748,26 +2758,28 @@
       <x:c r="I62" s="5" t="n">
         <x:v>46274.5</x:v>
       </x:c>
-      <x:c r="J62" s="4" t="str"/>
+      <x:c r="J62" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="14" t="str">
-        <x:v>E-08</x:v>
+        <x:v>D-16</x:v>
       </x:c>
       <x:c r="B63" s="3" t="str">
-        <x:v>Miro-app og UI</x:v>
+        <x:v>Sticky → Jira</x:v>
       </x:c>
       <x:c r="C63" s="3" t="str">
-        <x:v>Kortmeny</x:v>
+        <x:v>Direkte Jira-sak samtidig</x:v>
       </x:c>
       <x:c r="D63" s="4" t="str">
-        <x:v>Åpne menyen på et Jira-kort og velg kommentarer/lukk.</x:v>
+        <x:v>Opprett Jira-sak direkte mens sticky-konvertering skjer.</x:v>
       </x:c>
       <x:c r="E63" s="4" t="str">
-        <x:v>Riktig issueKey sendes til modal, og lukk fungerer.</x:v>
+        <x:v>Direkte Jira-sak går til Incoming; sticky-opprinnelig sak lager ikke ekstra Incoming-card.</x:v>
       </x:c>
       <x:c r="F63" s="4" t="str">
-        <x:v>Miro UI</x:v>
+        <x:v>Miro-board</x:v>
       </x:c>
       <x:c r="G63" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2784,22 +2796,22 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="14" t="str">
-        <x:v>F-01</x:v>
+        <x:v>E-01</x:v>
       </x:c>
       <x:c r="B64" s="3" t="str">
-        <x:v>Reliabilitet</x:v>
+        <x:v>Miro-app og UI</x:v>
       </x:c>
       <x:c r="C64" s="3" t="str">
-        <x:v>Queue-forsinkelse</x:v>
+        <x:v>App åpnes</x:v>
       </x:c>
       <x:c r="D64" s="4" t="str">
-        <x:v>Gjennomfør minst fem statusendringer og noter total tid.</x:v>
+        <x:v>Åpne Miro-appen og klikk appikon/panel.</x:v>
       </x:c>
       <x:c r="E64" s="4" t="str">
-        <x:v>Webhook køres én gang per event, og ingen hendelser blir hengende.</x:v>
+        <x:v>Panel åpnes, eksisterende kort oppdages, og /health er tilgjengelig.</x:v>
       </x:c>
       <x:c r="F64" s="4" t="str">
-        <x:v>Cloudflare queue</x:v>
+        <x:v>Miro UI</x:v>
       </x:c>
       <x:c r="G64" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2816,74 +2828,84 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="14" t="str">
-        <x:v>F-02</x:v>
+        <x:v>E-02</x:v>
       </x:c>
       <x:c r="B65" s="3" t="str">
-        <x:v>Reliabilitet</x:v>
+        <x:v>Miro-app og UI</x:v>
       </x:c>
       <x:c r="C65" s="3" t="str">
-        <x:v>Tregt Miro-kall</x:v>
+        <x:v>Custom-card registrering</x:v>
       </x:c>
       <x:c r="D65" s="4" t="str">
-        <x:v>Gjennomfør statusendring når Miro svarer tregt.</x:v>
+        <x:v>Åpne board med eksisterende custom cards.</x:v>
       </x:c>
       <x:c r="E65" s="4" t="str">
-        <x:v>Sync feiler ikke stille; resultatet blir korrekt og retry gir ikke duplikat.</x:v>
+        <x:v>Custom-card Jira-lenker og mappings registreres uten duplikat.</x:v>
       </x:c>
       <x:c r="F65" s="4" t="str">
-        <x:v>Cloudflare og Miro-board</x:v>
+        <x:v>Miro-board og CARD_MAP</x:v>
       </x:c>
       <x:c r="G65" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H65" s="3" t="str"/>
-      <x:c r="I65" s="5" t="str"/>
-      <x:c r="J65" s="4" t="str"/>
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H65" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I65" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J65" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="14" t="str">
-        <x:v>F-03</x:v>
+        <x:v>E-03</x:v>
       </x:c>
       <x:c r="B66" s="3" t="str">
-        <x:v>Reliabilitet</x:v>
+        <x:v>Miro-app og UI</x:v>
       </x:c>
       <x:c r="C66" s="3" t="str">
-        <x:v>HTTP 500/retry</x:v>
+        <x:v>Jira-link på native-card</x:v>
       </x:c>
       <x:c r="D66" s="4" t="str">
-        <x:v>Fremprovoser en Miro/Jira 500 i testmiljø.</x:v>
+        <x:v>Klikk Jira-lenken på et native Jira-kort.</x:v>
       </x:c>
       <x:c r="E66" s="4" t="str">
-        <x:v>Feil blir synlig, queue retry skjer innen konfigurerte grenser, og systemet stabiliserer seg.</x:v>
+        <x:v>Lenken åpner riktig Jira-sak i riktig site/prosjekt.</x:v>
       </x:c>
       <x:c r="F66" s="4" t="str">
-        <x:v>Cloudflare queue</x:v>
+        <x:v>Ikke relevant: løsningen bruker kun custom cards.</x:v>
       </x:c>
       <x:c r="G66" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H66" s="3" t="str"/>
-      <x:c r="I66" s="5" t="str"/>
+        <x:v>Ikke relevant</x:v>
+      </x:c>
+      <x:c r="H66" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I66" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
       <x:c r="J66" s="4" t="str"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="14" t="str">
-        <x:v>F-04</x:v>
+        <x:v>E-04</x:v>
       </x:c>
       <x:c r="B67" s="3" t="str">
-        <x:v>Reliabilitet</x:v>
+        <x:v>Miro-app og UI</x:v>
       </x:c>
       <x:c r="C67" s="3" t="str">
-        <x:v>Refresh etter deploy</x:v>
+        <x:v>Jira-link på custom-card</x:v>
       </x:c>
       <x:c r="D67" s="4" t="str">
-        <x:v>Refresh Miro og åpne appen på nytt etter deploy.</x:v>
+        <x:v>Klikk Jira-lenken på et custom-kort.</x:v>
       </x:c>
       <x:c r="E67" s="4" t="str">
-        <x:v>Appen registrerer kort, mappings og indikatorer på nytt uten duplikater.</x:v>
+        <x:v>Lenken åpner riktig Jira-sak i riktig site/prosjekt.</x:v>
       </x:c>
       <x:c r="F67" s="4" t="str">
-        <x:v>Miro UI og CARD_MAP</x:v>
+        <x:v>Nettleser og Jira-URL</x:v>
       </x:c>
       <x:c r="G67" s="3" t="str">
         <x:v>Bestått</x:v>
@@ -2900,66 +2922,306 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="14" t="str">
+        <x:v>E-05</x:v>
+      </x:c>
+      <x:c r="B68" s="3" t="str">
+        <x:v>Miro-app og UI</x:v>
+      </x:c>
+      <x:c r="C68" s="3" t="str">
+        <x:v>Jira-link etter refresh</x:v>
+      </x:c>
+      <x:c r="D68" s="4" t="str">
+        <x:v>Refresh Miro, åpne boardet på nytt og klikk lenken på et custom-kort.</x:v>
+      </x:c>
+      <x:c r="E68" s="4" t="str">
+        <x:v>Lenken er fortsatt til stede og peker til riktig Jira-sak.</x:v>
+      </x:c>
+      <x:c r="F68" s="4" t="str">
+        <x:v>Miro-board og Jira-URL</x:v>
+      </x:c>
+      <x:c r="G68" s="3" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H68" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I68" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J68" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="14" t="str">
+        <x:v>E-06</x:v>
+      </x:c>
+      <x:c r="B69" s="3" t="str">
+        <x:v>Miro-app og UI</x:v>
+      </x:c>
+      <x:c r="C69" s="3" t="str">
+        <x:v>Legacy group-opprydding</x:v>
+      </x:c>
+      <x:c r="D69" s="4" t="str">
+        <x:v>Test av gammel native-card/grupperingslogikk.</x:v>
+      </x:c>
+      <x:c r="E69" s="4" t="str">
+        <x:v>Ikke relevant: løsningen bruker kun custom cards.</x:v>
+      </x:c>
+      <x:c r="F69" s="4" t="str">
+        <x:v>Ikke relevant: native Jira cards brukes ikke.</x:v>
+      </x:c>
+      <x:c r="G69" s="3" t="str">
+        <x:v>Ikke relevant</x:v>
+      </x:c>
+      <x:c r="H69" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I69" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J69" s="4" t="str"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="14" t="str">
+        <x:v>E-07</x:v>
+      </x:c>
+      <x:c r="B70" s="3" t="str">
+        <x:v>Miro-app og UI</x:v>
+      </x:c>
+      <x:c r="C70" s="3" t="str">
+        <x:v>Kommentarindikator følger kort</x:v>
+      </x:c>
+      <x:c r="D70" s="4" t="str">
+        <x:v>Test av gammel kort-/indikatorflyt.</x:v>
+      </x:c>
+      <x:c r="E70" s="4" t="str">
+        <x:v>Ikke relevant: denne flyten inngår ikke i ønsket custom-card-testomfang.</x:v>
+      </x:c>
+      <x:c r="F70" s="4" t="str">
+        <x:v>Ikke relevant: utenfor avtalt testomfang.</x:v>
+      </x:c>
+      <x:c r="G70" s="3" t="str">
+        <x:v>Ikke relevant</x:v>
+      </x:c>
+      <x:c r="H70" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I70" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J70" s="4" t="str"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="14" t="str">
+        <x:v>E-08</x:v>
+      </x:c>
+      <x:c r="B71" s="3" t="str">
+        <x:v>Miro-app og UI</x:v>
+      </x:c>
+      <x:c r="C71" s="3" t="str">
+        <x:v>Kortmeny</x:v>
+      </x:c>
+      <x:c r="D71" s="4" t="str">
+        <x:v>Åpne menyen på et Jira-kort og velg kommentarer/lukk.</x:v>
+      </x:c>
+      <x:c r="E71" s="4" t="str">
+        <x:v>Riktig issueKey sendes til modal, og lukk fungerer.</x:v>
+      </x:c>
+      <x:c r="F71" s="4" t="str">
+        <x:v>Miro UI</x:v>
+      </x:c>
+      <x:c r="G71" s="3" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H71" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I71" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J71" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="14" t="str">
+        <x:v>F-01</x:v>
+      </x:c>
+      <x:c r="B72" s="3" t="str">
+        <x:v>Reliabilitet</x:v>
+      </x:c>
+      <x:c r="C72" s="3" t="str">
+        <x:v>Queue-forsinkelse</x:v>
+      </x:c>
+      <x:c r="D72" s="4" t="str">
+        <x:v>Gjennomfør minst fem statusendringer og noter total tid.</x:v>
+      </x:c>
+      <x:c r="E72" s="4" t="str">
+        <x:v>Webhook køres én gang per event, og ingen hendelser blir hengende.</x:v>
+      </x:c>
+      <x:c r="F72" s="4" t="str">
+        <x:v>Cloudflare queue</x:v>
+      </x:c>
+      <x:c r="G72" s="3" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H72" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I72" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J72" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="14" t="str">
+        <x:v>F-02</x:v>
+      </x:c>
+      <x:c r="B73" s="3" t="str">
+        <x:v>Reliabilitet</x:v>
+      </x:c>
+      <x:c r="C73" s="3" t="str">
+        <x:v>Tregt Miro-kall</x:v>
+      </x:c>
+      <x:c r="D73" s="4" t="str">
+        <x:v>Gjennomfør statusendring når Miro svarer tregt.</x:v>
+      </x:c>
+      <x:c r="E73" s="4" t="str">
+        <x:v>Sync feiler ikke stille; resultatet blir korrekt og retry gir ikke duplikat.</x:v>
+      </x:c>
+      <x:c r="F73" s="4" t="str">
+        <x:v>Cloudflare og Miro-board</x:v>
+      </x:c>
+      <x:c r="G73" s="3" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H73" s="3" t="str"/>
+      <x:c r="I73" s="5" t="str"/>
+      <x:c r="J73" s="4" t="str"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="14" t="str">
+        <x:v>F-03</x:v>
+      </x:c>
+      <x:c r="B74" s="3" t="str">
+        <x:v>Reliabilitet</x:v>
+      </x:c>
+      <x:c r="C74" s="3" t="str">
+        <x:v>HTTP 500/retry</x:v>
+      </x:c>
+      <x:c r="D74" s="4" t="str">
+        <x:v>Fremprovoser en Miro/Jira 500 i testmiljø.</x:v>
+      </x:c>
+      <x:c r="E74" s="4" t="str">
+        <x:v>Feil blir synlig, queue retry skjer innen konfigurerte grenser, og systemet stabiliserer seg.</x:v>
+      </x:c>
+      <x:c r="F74" s="4" t="str">
+        <x:v>Cloudflare queue</x:v>
+      </x:c>
+      <x:c r="G74" s="3" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="H74" s="3" t="str"/>
+      <x:c r="I74" s="5" t="str"/>
+      <x:c r="J74" s="4" t="str"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="14" t="str">
+        <x:v>F-04</x:v>
+      </x:c>
+      <x:c r="B75" s="3" t="str">
+        <x:v>Reliabilitet</x:v>
+      </x:c>
+      <x:c r="C75" s="3" t="str">
+        <x:v>Refresh etter deploy</x:v>
+      </x:c>
+      <x:c r="D75" s="4" t="str">
+        <x:v>Refresh Miro og åpne appen på nytt etter deploy.</x:v>
+      </x:c>
+      <x:c r="E75" s="4" t="str">
+        <x:v>Appen registrerer kort, mappings og indikatorer på nytt uten duplikater.</x:v>
+      </x:c>
+      <x:c r="F75" s="4" t="str">
+        <x:v>Miro UI og CARD_MAP</x:v>
+      </x:c>
+      <x:c r="G75" s="3" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H75" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I75" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J75" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="14" t="str">
         <x:v>F-05</x:v>
       </x:c>
-      <x:c r="B68" s="3" t="str">
+      <x:c r="B76" s="3" t="str">
         <x:v>Reliabilitet</x:v>
       </x:c>
-      <x:c r="C68" s="3" t="str">
+      <x:c r="C76" s="3" t="str">
         <x:v>Full statusrunde</x:v>
       </x:c>
-      <x:c r="D68" s="4" t="str">
+      <x:c r="D76" s="4" t="str">
         <x:v>Kjør én sak gjennom alle godkjente Jira-statuser og tilbake via Miro.</x:v>
       </x:c>
-      <x:c r="E68" s="4" t="str">
+      <x:c r="E76" s="4" t="str">
         <x:v>Jira og Miro ender med samme status hele veien.</x:v>
       </x:c>
-      <x:c r="F68" s="4" t="str">
+      <x:c r="F76" s="4" t="str">
         <x:v>Jira og Miro-board</x:v>
       </x:c>
-      <x:c r="G68" s="3" t="str">
-        <x:v>Bestått</x:v>
-      </x:c>
-      <x:c r="H68" s="3" t="str">
-        <x:v>Terje</x:v>
-      </x:c>
-      <x:c r="I68" s="5" t="n">
-        <x:v>46274.5</x:v>
-      </x:c>
-      <x:c r="J68" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69" s="2"/>
-      <x:c r="B69" s="2"/>
-      <x:c r="C69" s="2"/>
-      <x:c r="D69" s="2"/>
-      <x:c r="E69" s="2"/>
-      <x:c r="F69" s="2"/>
-      <x:c r="G69" s="2"/>
-      <x:c r="H69" s="2"/>
-      <x:c r="I69" s="2"/>
-      <x:c r="J69" s="2"/>
+      <x:c r="G76" s="3" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H76" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I76" s="5" t="n">
+        <x:v>46274.5</x:v>
+      </x:c>
+      <x:c r="J76" s="4" t="str">
+        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="2"/>
+      <x:c r="B77" s="2"/>
+      <x:c r="C77" s="2"/>
+      <x:c r="D77" s="2"/>
+      <x:c r="E77" s="2"/>
+      <x:c r="F77" s="2"/>
+      <x:c r="G77" s="2"/>
+      <x:c r="H77" s="2"/>
+      <x:c r="I77" s="2"/>
+      <x:c r="J77" s="2"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G5:G68">
+  <x:conditionalFormatting sqref="G5:G76">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Bestått"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Feilet"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Blokkert"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="G5:G68">
+    <x:dataValidation type="list" sqref="G5:G76">
       <x:formula1>"Ikke testet,Bestått,Feilet,Blokkert,Ikke relevant"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4611015adfe4b9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rade77bffed2d4b33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3110,134 +3372,727 @@
         <x:v>Miro custom-card create/refresh/dedupe</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>B-01, B-02, B-09–B-11, B-15–B-16, D-01–D-16</x:v>
+        <x:v>B-01, B-02, B-09–B-11, B-15–B-21, D-01–D-16</x:v>
       </x:c>
       <x:c r="C13" s="31" t="str">
-        <x:v>Card-innhold, duplikatkontroll og posisjon</x:v>
+        <x:v>Card-innhold, duplikatkontroll, visuelle regler og posisjon</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30" t="str">
-        <x:v>Miro mapping og Incoming</x:v>
+        <x:v>Custom-card visuelle regler</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>B-01–B-02, B-15–B-16, E-02</x:v>
+        <x:v>B-10, B-18–B-21</x:v>
       </x:c>
       <x:c r="C14" s="31" t="str">
-        <x:v>CARD_MAP, Incoming og stale mapping</x:v>
+        <x:v>Blocker-sort, Hotfix-felt, work type-farger og prioritetsikoner</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="30" t="str">
-        <x:v>Collision/placement</x:v>
+        <x:v>Miro mapping og Incoming</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>C-05, C-10, D-01–D-06</x:v>
+        <x:v>B-01–B-02, B-15–B-16, E-02</x:v>
       </x:c>
       <x:c r="C15" s="31" t="str">
-        <x:v>Y-bevaring, kolonnegrense og kollisjonsfri plassering</x:v>
+        <x:v>CARD_MAP, Incoming og stale mapping</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="30" t="str">
-        <x:v>Parent-cache</x:v>
+        <x:v>Collision/placement</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>B-17, F-04</x:v>
+        <x:v>C-05, C-10, D-01–D-06</x:v>
       </x:c>
       <x:c r="C16" s="31" t="str">
-        <x:v>Cache ved varm instans og korrekt oppførsel etter refresh/deploy</x:v>
+        <x:v>Y-bevaring, kolonnegrense og kollisjonsfri plassering</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="30" t="str">
-        <x:v>src/app-client.js: drag/debounce</x:v>
+        <x:v>Parent-cache</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>C-02–C-11, E-02–E-08</x:v>
+        <x:v>B-17, F-04</x:v>
       </x:c>
       <x:c r="C17" s="31" t="str">
-        <x:v>Custom-card-drag, 60 %-regel, debounce, statuskall og link/UI-flyt</x:v>
+        <x:v>Cache ved varm instans og korrekt oppførsel etter refresh/deploy</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="str">
-        <x:v>Miro rollback og varsler</x:v>
+        <x:v>src/app-client.js: drag/debounce</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>C-07–C-08, D-14</x:v>
+        <x:v>C-02–C-11, E-02–E-08</x:v>
       </x:c>
       <x:c r="C18" s="31" t="str">
-        <x:v>Tilbakerulling ved Jira-feil</x:v>
+        <x:v>Custom-card-drag, 60 %-regel, debounce, statuskall og link/UI-flyt</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30" t="str">
-        <x:v>Kommentarindikator og kortmeny</x:v>
+        <x:v>Miro rollback og varsler</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>B-12–B-13, C-12–C-13, E-04–E-05</x:v>
+        <x:v>C-07–C-08, D-14</x:v>
       </x:c>
       <x:c r="C19" s="31" t="str">
-        <x:v>Indikator, følgeposisjon og modal</x:v>
+        <x:v>Tilbakerulling ved Jira-feil</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="30" t="str">
-        <x:v>Sticky-posisjon og workflow</x:v>
+        <x:v>Kommentarindikator og kortmeny</x:v>
       </x:c>
       <x:c r="B20" s="24" t="str">
-        <x:v>D-01–D-06, D-14–D-16</x:v>
+        <x:v>B-12–B-13, C-12–C-13, E-04–E-05</x:v>
       </x:c>
       <x:c r="C20" s="31" t="str">
-        <x:v>Eksakt posisjon, status og feilisolering</x:v>
+        <x:v>Indikator, følgeposisjon og modal</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="30" t="str">
-        <x:v>Sticky idempotens og metadata</x:v>
+        <x:v>Sticky-posisjon og workflow</x:v>
       </x:c>
       <x:c r="B21" s="24" t="str">
-        <x:v>D-11–D-13, D-16</x:v>
+        <x:v>D-01–D-06, D-14–D-16</x:v>
       </x:c>
       <x:c r="C21" s="31" t="str">
-        <x:v>Reporter, retry og konkurrerende Jira-webhook</x:v>
+        <x:v>Eksakt posisjon, status og feilisolering</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="30" t="str">
-        <x:v>src/panel-client.js: panel og multi-select</x:v>
+        <x:v>Sticky idempotens og metadata</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
-        <x:v>D-01–D-16, E-01</x:v>
+        <x:v>D-11–D-13, D-16</x:v>
       </x:c>
       <x:c r="C22" s="31" t="str">
-        <x:v>Konvertering, work type og fortsettelse etter feil</x:v>
+        <x:v>Reporter, retry og konkurrerende Jira-webhook</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="30" t="str">
+        <x:v>src/panel-client.js: panel og multi-select</x:v>
+      </x:c>
+      <x:c r="B23" s="24" t="str">
+        <x:v>D-01–D-16, E-01</x:v>
+      </x:c>
+      <x:c r="C23" s="31" t="str">
+        <x:v>Konvertering, work type og fortsettelse etter feil</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="30" t="str">
         <x:v>src/ui.js / comments-client.js</x:v>
       </x:c>
-      <x:c r="B23" s="24" t="str">
+      <x:c r="B24" s="24" t="str">
         <x:v>C-12–C-13, E-01, E-03–E-05, E-08</x:v>
       </x:c>
-      <x:c r="C23" s="31" t="str">
+      <x:c r="C24" s="31" t="str">
         <x:v>Modaler, panel, Jira-lenker og brukerflyt</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="32" t="str">
+    <x:row r="25">
+      <x:c r="A25" s="32" t="str">
         <x:v>Drift, observability og queue</x:v>
       </x:c>
-      <x:c r="B24" s="33" t="str">
+      <x:c r="B25" s="33" t="str">
         <x:v>F-01–F-05</x:v>
       </x:c>
-      <x:c r="C24" s="34" t="str">
+      <x:c r="C25" s="34" t="str">
         <x:v>Queue delay, treghet, 500, retry og deploy-refresh</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="27" t="str">
+        <x:v>Kilde</x:v>
+      </x:c>
+      <x:c r="B1" s="28" t="str">
+        <x:v>Funksjon</x:v>
+      </x:c>
+      <x:c r="C1" s="28" t="str">
+        <x:v>Test-ID</x:v>
+      </x:c>
+      <x:c r="D1" s="28" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="str">
+        <x:v>Hva verifiseres</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="20" t="str">
+        <x:v>src/index.js</x:v>
+      </x:c>
+      <x:c r="B2" s="24" t="str">
+        <x:v>GET /health</x:v>
+      </x:c>
+      <x:c r="C2" s="24" t="str">
+        <x:v>A-01</x:v>
+      </x:c>
+      <x:c r="D2" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E2" s="31" t="str">
+        <x:v>Konfigurasjon og nødvendige bindings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="20" t="str">
+        <x:v>src/auth.js</x:v>
+      </x:c>
+      <x:c r="B3" s="24" t="str">
+        <x:v>OPTIONS/CORS</x:v>
+      </x:c>
+      <x:c r="C3" s="24" t="str">
+        <x:v>A-02</x:v>
+      </x:c>
+      <x:c r="D3" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E3" s="31" t="str">
+        <x:v>Preflight-headere og tillatte metoder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="20" t="str">
+        <x:v>src/ui.js / app-client.js</x:v>
+      </x:c>
+      <x:c r="B4" s="24" t="str">
+        <x:v>Miro-app åpnes og registrerer custom cards</x:v>
+      </x:c>
+      <x:c r="C4" s="24" t="str">
+        <x:v>E-01, E-02</x:v>
+      </x:c>
+      <x:c r="D4" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E4" s="31" t="str">
+        <x:v>Panel, health og mapping-registrering</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="20" t="str">
+        <x:v>src/auth.js</x:v>
+      </x:c>
+      <x:c r="B5" s="24" t="str">
+        <x:v>Miro-token valideres</x:v>
+      </x:c>
+      <x:c r="C5" s="24" t="str">
+        <x:v>A-03</x:v>
+      </x:c>
+      <x:c r="D5" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E5" s="31" t="str">
+        <x:v>Beskyttede routes avviser ugyldig token</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="20" t="str">
+        <x:v>src/auth.js / index.js</x:v>
+      </x:c>
+      <x:c r="B6" s="24" t="str">
+        <x:v>Jira-webhook secret, prosjektfilter og HMAC</x:v>
+      </x:c>
+      <x:c r="C6" s="24" t="str">
+        <x:v>A-04, A-05, B-13</x:v>
+      </x:c>
+      <x:c r="D6" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E6" s="31" t="str">
+        <x:v>Ugyldige og godkjente webhooker</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="20" t="str">
+        <x:v>src/index.js</x:v>
+      </x:c>
+      <x:c r="B7" s="24" t="str">
+        <x:v>Ugyldig JSON og obligatoriske felter</x:v>
+      </x:c>
+      <x:c r="C7" s="24" t="str">
+        <x:v>A-06</x:v>
+      </x:c>
+      <x:c r="D7" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E7" s="31" t="str">
+        <x:v>Kontrollerte 400-responser uten sideeffekt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="20" t="str">
+        <x:v>src/index.js</x:v>
+      </x:c>
+      <x:c r="B8" s="24" t="str">
+        <x:v>Feil board, feil mapping og route-eierskap</x:v>
+      </x:c>
+      <x:c r="C8" s="24" t="str">
+        <x:v>A-07</x:v>
+      </x:c>
+      <x:c r="D8" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E8" s="31" t="str">
+        <x:v>403 ved uautorisert Miro/Jira-kobling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="20" t="str">
+        <x:v>src/index.js</x:v>
+      </x:c>
+      <x:c r="B9" s="24" t="str">
+        <x:v>Ukjent route eller HTTP-metode</x:v>
+      </x:c>
+      <x:c r="C9" s="24" t="str">
+        <x:v>A-08</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E9" s="31" t="str">
+        <x:v>404 uten sideeffekt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="20" t="str">
+        <x:v>src/index.js</x:v>
+      </x:c>
+      <x:c r="B10" s="24" t="str">
+        <x:v>Ugyldig issueKey, status eller posisjon</x:v>
+      </x:c>
+      <x:c r="C10" s="24" t="str">
+        <x:v>A-09</x:v>
+      </x:c>
+      <x:c r="D10" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E10" s="31" t="str">
+        <x:v>Kontrollert avvisning/ignorering</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="20" t="str">
+        <x:v>src/index.js / cards.js</x:v>
+      </x:c>
+      <x:c r="B11" s="24" t="str">
+        <x:v>Ny Jira-sak til Incoming custom card</x:v>
+      </x:c>
+      <x:c r="C11" s="24" t="str">
+        <x:v>B-01</x:v>
+      </x:c>
+      <x:c r="D11" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E11" s="31" t="str">
+        <x:v>Én card, dedupe og riktig mapping</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="20" t="str">
+        <x:v>src/app-client.js / index.js</x:v>
+      </x:c>
+      <x:c r="B12" s="24" t="str">
+        <x:v>Mapping-registrering, stale mapping og recovery</x:v>
+      </x:c>
+      <x:c r="C12" s="24" t="str">
+        <x:v>B-15, E-02</x:v>
+      </x:c>
+      <x:c r="D12" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E12" s="31" t="str">
+        <x:v>CARD_MAP og board-søk</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="20" t="str">
+        <x:v>src/index.js / miro.js</x:v>
+      </x:c>
+      <x:c r="B13" s="24" t="str">
+        <x:v>Jira-status flytter kortet gjennom workflow</x:v>
+      </x:c>
+      <x:c r="C13" s="24" t="str">
+        <x:v>B-03, B-04, B-05, B-06, B-07, F-05</x:v>
+      </x:c>
+      <x:c r="D13" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E13" s="31" t="str">
+        <x:v>X-flytting og Y-bevaring</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="20" t="str">
+        <x:v>src/cards.js / jira.js</x:v>
+      </x:c>
+      <x:c r="B14" s="24" t="str">
+        <x:v>Summary, priority og assignee refresher card</x:v>
+      </x:c>
+      <x:c r="C14" s="24" t="str">
+        <x:v>B-09, B-10, B-11</x:v>
+      </x:c>
+      <x:c r="D14" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E14" s="31" t="str">
+        <x:v>SVG-innhold oppdateres uten duplikat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="20" t="str">
+        <x:v>src/cards.js</x:v>
+      </x:c>
+      <x:c r="B15" s="24" t="str">
+        <x:v>Blocker-prioritet gjør kortet svart</x:v>
+      </x:c>
+      <x:c r="C15" s="24" t="str">
+        <x:v>B-18</x:v>
+      </x:c>
+      <x:c r="D15" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E15" s="31" t="str">
+        <x:v>Svart bakgrunn, hvit tekst og lesbar Jira-lenke</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="20" t="str">
+        <x:v>src/cards.js / jira.js</x:v>
+      </x:c>
+      <x:c r="B16" s="24" t="str">
+        <x:v>Hotfix-felt gjør kortet oransje</x:v>
+      </x:c>
+      <x:c r="C16" s="24" t="str">
+        <x:v>B-19</x:v>
+      </x:c>
+      <x:c r="D16" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E16" s="31" t="str">
+        <x:v>Hotfix-kort refresher til oransje</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="20" t="str">
+        <x:v>src/config.js / cards.js</x:v>
+      </x:c>
+      <x:c r="B17" s="24" t="str">
+        <x:v>Work type-farger</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="str">
+        <x:v>B-20</x:v>
+      </x:c>
+      <x:c r="D17" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E17" s="31" t="str">
+        <x:v>Bug, Improvement, Spike, New Feature og Task/config/doc/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="20" t="str">
+        <x:v>src/cards.js</x:v>
+      </x:c>
+      <x:c r="B18" s="24" t="str">
+        <x:v>Prioritetsikoner og prioritetstekst</x:v>
+      </x:c>
+      <x:c r="C18" s="24" t="str">
+        <x:v>B-10, B-21</x:v>
+      </x:c>
+      <x:c r="D18" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E18" s="31" t="str">
+        <x:v>Blocker/Highest/High/Medium/Low/Lowest/None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="20" t="str">
+        <x:v>src/cards.js / comments-client.js</x:v>
+      </x:c>
+      <x:c r="B19" s="24" t="str">
+        <x:v>Kommentarindikator ved opprettelse og sletting</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="str">
+        <x:v>B-12, B-13</x:v>
+      </x:c>
+      <x:c r="D19" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E19" s="31" t="str">
+        <x:v>Antall oppdateres og indikator fjernes ved null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="20" t="str">
+        <x:v>src/index.js / cards.js</x:v>
+      </x:c>
+      <x:c r="B20" s="24" t="str">
+        <x:v>Status-only webhook hopper over unødvendig SVG-refresh</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>B-08</x:v>
+      </x:c>
+      <x:c r="D20" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E20" s="31" t="str">
+        <x:v>Kortet flyttes uten full refresh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="20" t="str">
+        <x:v>src/index.js / cards.js</x:v>
+      </x:c>
+      <x:c r="B21" s="24" t="str">
+        <x:v>Retry, idempotens og queue-feil</x:v>
+      </x:c>
+      <x:c r="C21" s="24" t="str">
+        <x:v>B-16, D-13, F-02, F-03</x:v>
+      </x:c>
+      <x:c r="D21" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E21" s="31" t="str">
+        <x:v>Ingen duplikat og synlig feil ved retry/500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="20" t="str">
+        <x:v>src/index.js</x:v>
+      </x:c>
+      <x:c r="B22" s="24" t="str">
+        <x:v>Parent-cache og raske gjentatte statuser</x:v>
+      </x:c>
+      <x:c r="C22" s="24" t="str">
+        <x:v>B-17</x:v>
+      </x:c>
+      <x:c r="D22" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E22" s="31" t="str">
+        <x:v>Korrekt varm-cache og resultat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="20" t="str">
+        <x:v>src/app-client.js / index.js / jira.js</x:v>
+      </x:c>
+      <x:c r="B23" s="24" t="str">
+        <x:v>Custom card drag til Jira-status</x:v>
+      </x:c>
+      <x:c r="C23" s="24" t="str">
+        <x:v>C-02, C-03, C-04, C-05, C-06, C-10, C-11</x:v>
+      </x:c>
+      <x:c r="D23" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E23" s="31" t="str">
+        <x:v>60 %-regel, debounce og kollisjon</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="20" t="str">
+        <x:v>src/app-client.js / jira.js</x:v>
+      </x:c>
+      <x:c r="B24" s="24" t="str">
+        <x:v>Jira-avvisning, rollback og Test area-gate</x:v>
+      </x:c>
+      <x:c r="C24" s="24" t="str">
+        <x:v>C-07, C-08, C-09, D-14</x:v>
+      </x:c>
+      <x:c r="D24" s="24" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E24" s="31" t="str">
+        <x:v>Kort tilbake, melding og gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="20" t="str">
+        <x:v>src/index.js / comments-client.js</x:v>
+      </x:c>
+      <x:c r="B25" s="24" t="str">
+        <x:v>Les og opprett Jira-kommentar fra Miro</x:v>
+      </x:c>
+      <x:c r="C25" s="24" t="str">
+        <x:v>C-12, C-13</x:v>
+      </x:c>
+      <x:c r="D25" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E25" s="31" t="str">
+        <x:v>Riktig sak, bruker og validering</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="20" t="str">
+        <x:v>src/panel-client.js / jira.js</x:v>
+      </x:c>
+      <x:c r="B26" s="24" t="str">
+        <x:v>Sticky-konvertering og eksakt posisjon</x:v>
+      </x:c>
+      <x:c r="C26" s="24" t="str">
+        <x:v>D-01, D-02, D-03, D-04, D-05, D-06</x:v>
+      </x:c>
+      <x:c r="D26" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E26" s="31" t="str">
+        <x:v>Sak, card, status og posisjon</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="20" t="str">
+        <x:v>src/jira.js</x:v>
+      </x:c>
+      <x:c r="B27" s="24" t="str">
+        <x:v>Work type og obligatoriske sticky-defaults</x:v>
+      </x:c>
+      <x:c r="C27" s="24" t="str">
+        <x:v>D-07, D-08, D-09, D-10</x:v>
+      </x:c>
+      <x:c r="D27" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E27" s="31" t="str">
+        <x:v>Bug, Improvement, New Feature og Task/config/doc/test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="20" t="str">
+        <x:v>src/jira.js</x:v>
+      </x:c>
+      <x:c r="B28" s="24" t="str">
+        <x:v>Reporter og Original Miro created metadata</x:v>
+      </x:c>
+      <x:c r="C28" s="24" t="str">
+        <x:v>D-11, D-12</x:v>
+      </x:c>
+      <x:c r="D28" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E28" s="31" t="str">
+        <x:v>Riktig bruker og tidspunkt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="20" t="str">
+        <x:v>src/panel-client.js</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Multi-select fortsetter etter individuell feil</x:v>
+      </x:c>
+      <x:c r="C29" s="24" t="str">
+        <x:v>D-15</x:v>
+      </x:c>
+      <x:c r="D29" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E29" s="31" t="str">
+        <x:v>Gyldige stickies konverteres videre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="20" t="str">
+        <x:v>src/index.js / config.js</x:v>
+      </x:c>
+      <x:c r="B30" s="24" t="str">
+        <x:v>Direkte Jira-sak samtidig med sticky-konvertering</x:v>
+      </x:c>
+      <x:c r="C30" s="24" t="str">
+        <x:v>D-16</x:v>
+      </x:c>
+      <x:c r="D30" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E30" s="31" t="str">
+        <x:v>Incoming og freeze-markører fungerer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="20" t="str">
+        <x:v>src/app-client.js</x:v>
+      </x:c>
+      <x:c r="B31" s="24" t="str">
+        <x:v>Jira-lenke på custom card og etter refresh</x:v>
+      </x:c>
+      <x:c r="C31" s="24" t="str">
+        <x:v>E-04, E-05</x:v>
+      </x:c>
+      <x:c r="D31" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E31" s="31" t="str">
+        <x:v>Lenke peker til riktig Jira-sak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="20" t="str">
+        <x:v>src/ui.js / app-client.js</x:v>
+      </x:c>
+      <x:c r="B32" s="24" t="str">
+        <x:v>Kortmeny og kommentarer-lenke</x:v>
+      </x:c>
+      <x:c r="C32" s="24" t="str">
+        <x:v>E-08</x:v>
+      </x:c>
+      <x:c r="D32" s="24" t="str">
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="E32" s="31" t="str">
+        <x:v>Riktig issueKey/itemId og lukk fungerer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="22" t="str">
+        <x:v>src/miro.js / cards.js</x:v>
+      </x:c>
+      <x:c r="B33" s="33" t="str">
+        <x:v>Slow Miro-kall, 500 og refresh etter deploy</x:v>
+      </x:c>
+      <x:c r="C33" s="33" t="str">
+        <x:v>F-02, F-03, F-04</x:v>
+      </x:c>
+      <x:c r="D33" s="33" t="str">
+        <x:v>Ikke testet</x:v>
+      </x:c>
+      <x:c r="E33" s="34" t="str">
+        <x:v>Feil, retry og registrering etter refresh</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="D2:D33">
+    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Bestått"/>
+    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Ikke testet"/>
+    <x:cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="Feilet"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update test report with Blocker verification
</commit_message>
<xml_diff>
--- a/docs/testing/jira-miro-full-test-plan.xlsx
+++ b/docs/testing/jira-miro-full-test-plan.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testoversikt" sheetId="1" r:id="R0f7bc65093a946c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testliste" sheetId="2" r:id="Ra1e8adb59e2f4e4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dekning" sheetId="3" r:id="R73e06116150a4f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funksjonsdekning" sheetId="4" r:id="R512d806e5df54e0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testoversikt" sheetId="1" r:id="R0342eb7e073448ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testliste" sheetId="2" r:id="R2889deedeac3490d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dekning" sheetId="3" r:id="R95eefc17f0e247a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funksjonsdekning" sheetId="4" r:id="Rd0c3b183394f408d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -219,7 +219,7 @@
         <x:color rgb="FF216E39"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -230,7 +230,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -241,7 +241,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -252,7 +252,7 @@
         <x:color rgb="FF216E39"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -263,7 +263,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -274,7 +274,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -584,7 +584,7 @@
       </x:c>
       <x:c r="B6" s="21" t="n">
         <x:f>COUNTIF(Testliste!$G$5:$G$76,"Bestått")</x:f>
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="20" t="str">
@@ -644,7 +644,7 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF(Testliste!$G$5:$G$76,"Ikke testet")</x:f>
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="20" t="str">
@@ -1163,15 +1163,19 @@
         <x:v>Kallet avvises med 403 og ingen Jira-endring skjer.</x:v>
       </x:c>
       <x:c r="F11" s="4" t="str">
-        <x:v>HTTP-respons og Jira-status</x:v>
+        <x:v>HTTP 403 mottatt ved feil boardId. Kallet ble avvist før Jira-statusendring.</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H11" s="3" t="str"/>
-      <x:c r="I11" s="5" t="str"/>
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I11" s="5" t="n">
+        <x:v>46275.260416666664</x:v>
+      </x:c>
       <x:c r="J11" s="4" t="str">
-        <x:v>Funnet ved funksjonsaudit. Krever egen negativ test.</x:v>
+        <x:v>Feil boardId ble avvist kontrollert.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1191,15 +1195,19 @@
         <x:v>Worker svarer 404 uten sideeffekter.</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>HTTP-respons</x:v>
+        <x:v>Ukjent route og feil HTTP-metode svarte med HTTP 404 Not Found.</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H12" s="3" t="str"/>
-      <x:c r="I12" s="5" t="str"/>
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I12" s="5" t="n">
+        <x:v>46275.270833333336</x:v>
+      </x:c>
       <x:c r="J12" s="4" t="str">
-        <x:v>Funnet ved funksjonsaudit. Krever egen negativ test.</x:v>
+        <x:v>Ingen Jira- eller Miro-endring.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1219,16 +1227,18 @@
         <x:v>Kallet avvises kontrollert eller ignoreres uten duplikat eller sideeffekt.</x:v>
       </x:c>
       <x:c r="F13" s="4" t="str">
-        <x:v>HTTP-respons og Miro-board</x:v>
+        <x:v>Ugyldig issueKey og posisjon ble avvist med HTTP 400. Ingen custom card ble opprettet eller flyttet.</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H13" s="3" t="str"/>
-      <x:c r="I13" s="5" t="str"/>
-      <x:c r="J13" s="4" t="str">
-        <x:v>Funnet ved funksjonsaudit. Krever egen negativ test.</x:v>
-      </x:c>
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I13" s="5" t="n">
+        <x:v>46275.28125</x:v>
+      </x:c>
+      <x:c r="J13" s="4" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14" t="str">
@@ -1545,7 +1555,7 @@
         <x:v>46274.5</x:v>
       </x:c>
       <x:c r="J23" s="4" t="str">
-        <x:v>Godkjent av bruker uten separat manuell test.</x:v>
+        <x:v>Low → Blocker verifisert. Custom-card ble oppdatert uten feil og ble svart med hvit tekst.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1788,12 +1798,16 @@
         <x:v>Miro-card</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
-        <x:v>Ikke testet</x:v>
-      </x:c>
-      <x:c r="H31" s="3" t="str"/>
-      <x:c r="I31" s="5" t="str"/>
+        <x:v>Bestått</x:v>
+      </x:c>
+      <x:c r="H31" s="3" t="str">
+        <x:v>Terje</x:v>
+      </x:c>
+      <x:c r="I31" s="5" t="n">
+        <x:v>46275.36666666667</x:v>
+      </x:c>
       <x:c r="J31" s="4" t="str">
-        <x:v>Funnet ved funksjonsaudit. Krever egen visuell test.</x:v>
+        <x:v>Prioritet endret fra Low til Blocker etter Spike → Bug. Custom-card ble svart, og Jira-lenken forble lesbar.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -1968,7 +1982,7 @@
         <x:v>Terje</x:v>
       </x:c>
       <x:c r="I37" s="5" t="n">
-        <x:v>46274.5</x:v>
+        <x:v>46275.36666666667</x:v>
       </x:c>
       <x:c r="J37" s="4" t="str">
         <x:v>Godkjent av bruker uten separat manuell test.</x:v>
@@ -3221,7 +3235,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rade77bffed2d4b33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcc102fc43da43d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3656,7 +3670,7 @@
         <x:v>A-07</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>Ikke testet</x:v>
+        <x:v>Bestått</x:v>
       </x:c>
       <x:c r="E8" s="31" t="str">
         <x:v>403 ved uautorisert Miro/Jira-kobling</x:v>
@@ -3673,7 +3687,7 @@
         <x:v>A-08</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
-        <x:v>Ikke testet</x:v>
+        <x:v>Bestått</x:v>
       </x:c>
       <x:c r="E9" s="31" t="str">
         <x:v>404 uten sideeffekt</x:v>
@@ -3690,7 +3704,7 @@
         <x:v>A-09</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
-        <x:v>Ikke testet</x:v>
+        <x:v>Bestått</x:v>
       </x:c>
       <x:c r="E10" s="31" t="str">
         <x:v>Kontrollert avvisning/ignorering</x:v>
@@ -3775,10 +3789,10 @@
         <x:v>B-18</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
-        <x:v>Ikke testet</x:v>
+        <x:v>Bestått</x:v>
       </x:c>
       <x:c r="E15" s="31" t="str">
-        <x:v>Svart bakgrunn, hvit tekst og lesbar Jira-lenke</x:v>
+        <x:v>Blocker-test gjennomført: kortet ble svart med hvit tekst, og Jira-lenken var fortsatt lesbar.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">

</xml_diff>